<commit_message>
modified:   R/notebooks/traverseaces.ipynb 	modified:   data/chapter2/FRED/subsets/species.xlsx 	modified:   notebooks/chapter_02/paper-draft.ipynb 	modified:   notebooks/chapter_02/phylogeney.ipynb
</commit_message>
<xml_diff>
--- a/data/chapter2/FRED/subsets/species.xlsx
+++ b/data/chapter2/FRED/subsets/species.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90963425_westernsydney_edu_au/Documents/PhD/code/data/chapter2/FRED/subsets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="156" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F734AB0-0C45-4A3B-B771-2EF4CB6A3323}"/>
+  <xr:revisionPtr revIDLastSave="170" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C16EE58C-132F-4521-95C6-CD00E34A73B7}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{A5444074-DC77-415C-A9E2-2BBA8270EAFC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{A5444074-DC77-415C-A9E2-2BBA8270EAFC}"/>
   </bookViews>
   <sheets>
     <sheet name="FRED4" sheetId="8" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3252" uniqueCount="1058">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3276" uniqueCount="1058">
   <si>
     <t>F00645</t>
   </si>
@@ -14835,7 +14835,9 @@
       <c r="B27" s="1" t="s">
         <v>947</v>
       </c>
-      <c r="C27" s="1"/>
+      <c r="C27" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
@@ -14844,7 +14846,9 @@
       <c r="B28" s="1" t="s">
         <v>944</v>
       </c>
-      <c r="C28" s="1"/>
+      <c r="C28" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
@@ -14853,7 +14857,9 @@
       <c r="B29" s="1" t="s">
         <v>945</v>
       </c>
-      <c r="C29" s="1"/>
+      <c r="C29" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
@@ -15016,7 +15022,9 @@
       <c r="B44" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C44" s="1"/>
+      <c r="C44" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
@@ -15025,7 +15033,9 @@
       <c r="B45" s="1" t="s">
         <v>945</v>
       </c>
-      <c r="C45" s="1"/>
+      <c r="C45" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
@@ -15034,7 +15044,9 @@
       <c r="B46" s="1" t="s">
         <v>945</v>
       </c>
-      <c r="C46" s="1"/>
+      <c r="C46" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
@@ -15043,7 +15055,9 @@
       <c r="B47" s="1" t="s">
         <v>947</v>
       </c>
-      <c r="C47" s="1"/>
+      <c r="C47" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
@@ -15052,7 +15066,9 @@
       <c r="B48" s="1" t="s">
         <v>951</v>
       </c>
-      <c r="C48" s="1"/>
+      <c r="C48" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
@@ -15061,7 +15077,9 @@
       <c r="B49" s="1" t="s">
         <v>951</v>
       </c>
-      <c r="C49" s="1"/>
+      <c r="C49" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
@@ -15634,7 +15652,9 @@
       <c r="B110" s="1" t="s">
         <v>951</v>
       </c>
-      <c r="C110" s="1"/>
+      <c r="C110" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
@@ -15643,7 +15663,9 @@
       <c r="B111" s="1" t="s">
         <v>951</v>
       </c>
-      <c r="C111" s="1"/>
+      <c r="C111" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
@@ -15652,7 +15674,9 @@
       <c r="B112" s="1" t="s">
         <v>947</v>
       </c>
-      <c r="C112" s="1"/>
+      <c r="C112" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
@@ -15661,7 +15685,9 @@
       <c r="B113" s="1" t="s">
         <v>951</v>
       </c>
-      <c r="C113" s="1"/>
+      <c r="C113" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
@@ -15670,7 +15696,9 @@
       <c r="B114" s="1" t="s">
         <v>947</v>
       </c>
-      <c r="C114" s="1"/>
+      <c r="C114" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
@@ -15679,7 +15707,9 @@
       <c r="B115" s="1" t="s">
         <v>951</v>
       </c>
-      <c r="C115" s="1"/>
+      <c r="C115" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
@@ -15688,7 +15718,9 @@
       <c r="B116" s="1" t="s">
         <v>947</v>
       </c>
-      <c r="C116" s="1"/>
+      <c r="C116" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
@@ -15697,7 +15729,9 @@
       <c r="B117" s="1" t="s">
         <v>947</v>
       </c>
-      <c r="C117" s="1"/>
+      <c r="C117" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
@@ -15706,7 +15740,9 @@
       <c r="B118" s="1" t="s">
         <v>951</v>
       </c>
-      <c r="C118" s="1"/>
+      <c r="C118" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
@@ -15715,7 +15751,9 @@
       <c r="B119" s="1" t="s">
         <v>951</v>
       </c>
-      <c r="C119" s="1"/>
+      <c r="C119" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
@@ -15742,7 +15780,9 @@
       <c r="B122" s="1" t="s">
         <v>951</v>
       </c>
-      <c r="C122" s="1"/>
+      <c r="C122" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
@@ -15751,7 +15791,9 @@
       <c r="B123" s="1" t="s">
         <v>951</v>
       </c>
-      <c r="C123" s="1"/>
+      <c r="C123" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
@@ -15760,7 +15802,9 @@
       <c r="B124" s="1" t="s">
         <v>951</v>
       </c>
-      <c r="C124" s="1"/>
+      <c r="C124" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
@@ -15769,7 +15813,9 @@
       <c r="B125" s="1" t="s">
         <v>951</v>
       </c>
-      <c r="C125" s="1"/>
+      <c r="C125" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
@@ -15778,7 +15824,9 @@
       <c r="B126" s="1" t="s">
         <v>947</v>
       </c>
-      <c r="C126" s="1"/>
+      <c r="C126" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A1048576">

</xml_diff>

<commit_message>
modified:   data/chapter2/FRED/subsets/species.xlsx 	new file:   data/chapter2/FRED/subsets/species_hand_cleaned.csv 	modified:   notebooks/chapter_02/paper-draft.ipynb
</commit_message>
<xml_diff>
--- a/data/chapter2/FRED/subsets/species.xlsx
+++ b/data/chapter2/FRED/subsets/species.xlsx
@@ -8,20 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90963425_westernsydney_edu_au/Documents/PhD/code/data/chapter2/FRED/subsets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="228" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A0F7066-243B-4F5A-A8C6-27417CE32066}"/>
+  <xr:revisionPtr revIDLastSave="307" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AFD6CD39-8D94-4943-82B9-80BFBF123A9A}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{A5444074-DC77-415C-A9E2-2BBA8270EAFC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{A5444074-DC77-415C-A9E2-2BBA8270EAFC}"/>
   </bookViews>
   <sheets>
     <sheet name="FRED4" sheetId="8" r:id="rId1"/>
     <sheet name="FungalRoot" sheetId="9" r:id="rId2"/>
-    <sheet name="Maherali 2016" sheetId="7" r:id="rId3"/>
+    <sheet name="Maherali_2016" sheetId="7" r:id="rId3"/>
     <sheet name="combined" sheetId="10" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="ExternalData_1" localSheetId="0" hidden="1">FRED4!$A$1:$B$936</definedName>
     <definedName name="ExternalData_1" localSheetId="1" hidden="1">FungalRoot!$A$1:$B$126</definedName>
-    <definedName name="ExternalData_1" localSheetId="2" hidden="1">'Maherali 2016'!$A$1:$B$70</definedName>
+    <definedName name="ExternalData_1" localSheetId="2" hidden="1">Maherali_2016!$A$1:$B$70</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -4583,7 +4583,7 @@
         <v>2</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
@@ -4594,7 +4594,7 @@
         <v>5</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
@@ -5595,7 +5595,7 @@
         <v>2</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.35">
@@ -5606,7 +5606,7 @@
         <v>5</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.35">
@@ -5716,7 +5716,7 @@
         <v>2</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.35">
@@ -5727,7 +5727,7 @@
         <v>5</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.35">
@@ -5760,7 +5760,7 @@
         <v>2</v>
       </c>
       <c r="C140" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.35">
@@ -5771,7 +5771,7 @@
         <v>5</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.35">
@@ -6112,7 +6112,7 @@
         <v>2</v>
       </c>
       <c r="C172" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.35">
@@ -6123,7 +6123,7 @@
         <v>5</v>
       </c>
       <c r="C173" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.35">
@@ -6211,7 +6211,7 @@
         <v>2</v>
       </c>
       <c r="C181" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.35">
@@ -6222,7 +6222,7 @@
         <v>5</v>
       </c>
       <c r="C182" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.35">
@@ -6453,7 +6453,7 @@
         <v>2</v>
       </c>
       <c r="C203" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.35">
@@ -6464,7 +6464,7 @@
         <v>5</v>
       </c>
       <c r="C204" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.35">
@@ -6519,7 +6519,7 @@
         <v>2</v>
       </c>
       <c r="C209" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.35">
@@ -6783,7 +6783,7 @@
         <v>2</v>
       </c>
       <c r="C233" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.35">
@@ -6794,7 +6794,7 @@
         <v>1</v>
       </c>
       <c r="C234" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.35">
@@ -6981,7 +6981,7 @@
         <v>1</v>
       </c>
       <c r="C251" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.35">
@@ -7003,7 +7003,7 @@
         <v>5</v>
       </c>
       <c r="C253" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.35">
@@ -7058,7 +7058,7 @@
         <v>2</v>
       </c>
       <c r="C258" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.35">
@@ -7069,7 +7069,7 @@
         <v>5</v>
       </c>
       <c r="C259" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.35">
@@ -7223,7 +7223,7 @@
         <v>2</v>
       </c>
       <c r="C273" s="1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.35">
@@ -7476,7 +7476,7 @@
         <v>2</v>
       </c>
       <c r="C296" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="297" spans="1:3" x14ac:dyDescent="0.35">
@@ -7487,7 +7487,7 @@
         <v>5</v>
       </c>
       <c r="C297" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="298" spans="1:3" x14ac:dyDescent="0.35">
@@ -7916,7 +7916,7 @@
         <v>5</v>
       </c>
       <c r="C336" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="337" spans="1:3" x14ac:dyDescent="0.35">
@@ -7927,7 +7927,7 @@
         <v>2</v>
       </c>
       <c r="C337" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="338" spans="1:3" x14ac:dyDescent="0.35">
@@ -7938,7 +7938,7 @@
         <v>2</v>
       </c>
       <c r="C338" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="339" spans="1:3" x14ac:dyDescent="0.35">
@@ -7949,7 +7949,7 @@
         <v>1</v>
       </c>
       <c r="C339" s="1" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="340" spans="1:3" x14ac:dyDescent="0.35">
@@ -7960,7 +7960,7 @@
         <v>5</v>
       </c>
       <c r="C340" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="341" spans="1:3" x14ac:dyDescent="0.35">
@@ -8092,7 +8092,7 @@
         <v>2</v>
       </c>
       <c r="C352" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="353" spans="1:3" x14ac:dyDescent="0.35">
@@ -8785,7 +8785,7 @@
         <v>5</v>
       </c>
       <c r="C415" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="416" spans="1:3" x14ac:dyDescent="0.35">
@@ -8796,7 +8796,7 @@
         <v>2</v>
       </c>
       <c r="C416" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="417" spans="1:3" x14ac:dyDescent="0.35">
@@ -8873,7 +8873,7 @@
         <v>2</v>
       </c>
       <c r="C423" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="424" spans="1:3" x14ac:dyDescent="0.35">
@@ -8928,7 +8928,7 @@
         <v>2</v>
       </c>
       <c r="C428" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="429" spans="1:3" x14ac:dyDescent="0.35">
@@ -8939,7 +8939,7 @@
         <v>5</v>
       </c>
       <c r="C429" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="430" spans="1:3" x14ac:dyDescent="0.35">
@@ -8972,7 +8972,7 @@
         <v>2</v>
       </c>
       <c r="C432" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="433" spans="1:3" x14ac:dyDescent="0.35">
@@ -8983,7 +8983,7 @@
         <v>1</v>
       </c>
       <c r="C433" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="434" spans="1:3" x14ac:dyDescent="0.35">
@@ -9115,7 +9115,7 @@
         <v>2</v>
       </c>
       <c r="C445" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="446" spans="1:3" x14ac:dyDescent="0.35">
@@ -9500,7 +9500,7 @@
         <v>1</v>
       </c>
       <c r="C480" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="481" spans="1:3" x14ac:dyDescent="0.35">
@@ -9511,7 +9511,7 @@
         <v>2</v>
       </c>
       <c r="C481" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="482" spans="1:3" x14ac:dyDescent="0.35">
@@ -9555,7 +9555,7 @@
         <v>2</v>
       </c>
       <c r="C485" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="486" spans="1:3" x14ac:dyDescent="0.35">
@@ -9566,7 +9566,7 @@
         <v>5</v>
       </c>
       <c r="C486" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="487" spans="1:3" x14ac:dyDescent="0.35">
@@ -10743,7 +10743,7 @@
         <v>2</v>
       </c>
       <c r="C593" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="594" spans="1:3" x14ac:dyDescent="0.35">
@@ -10754,7 +10754,7 @@
         <v>5</v>
       </c>
       <c r="C594" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="595" spans="1:3" x14ac:dyDescent="0.35">
@@ -10776,7 +10776,7 @@
         <v>1</v>
       </c>
       <c r="C596" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="597" spans="1:3" x14ac:dyDescent="0.35">
@@ -10787,7 +10787,7 @@
         <v>2</v>
       </c>
       <c r="C597" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="598" spans="1:3" x14ac:dyDescent="0.35">
@@ -10820,7 +10820,7 @@
         <v>1</v>
       </c>
       <c r="C600" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="601" spans="1:3" x14ac:dyDescent="0.35">
@@ -10831,7 +10831,7 @@
         <v>2</v>
       </c>
       <c r="C601" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="602" spans="1:3" x14ac:dyDescent="0.35">
@@ -11271,7 +11271,7 @@
         <v>2</v>
       </c>
       <c r="C641" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="642" spans="1:3" x14ac:dyDescent="0.35">
@@ -11282,7 +11282,7 @@
         <v>5</v>
       </c>
       <c r="C642" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="643" spans="1:3" x14ac:dyDescent="0.35">
@@ -11326,7 +11326,7 @@
         <v>2</v>
       </c>
       <c r="C646" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="647" spans="1:3" x14ac:dyDescent="0.35">
@@ -11337,7 +11337,7 @@
         <v>5</v>
       </c>
       <c r="C647" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="648" spans="1:3" x14ac:dyDescent="0.35">
@@ -11601,7 +11601,7 @@
         <v>5</v>
       </c>
       <c r="C671" s="1" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="672" spans="1:3" x14ac:dyDescent="0.35">
@@ -11733,7 +11733,7 @@
         <v>5</v>
       </c>
       <c r="C683" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="684" spans="1:3" x14ac:dyDescent="0.35">
@@ -11744,7 +11744,7 @@
         <v>1</v>
       </c>
       <c r="C684" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="685" spans="1:3" x14ac:dyDescent="0.35">
@@ -12316,7 +12316,7 @@
         <v>2</v>
       </c>
       <c r="C736" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="737" spans="1:3" x14ac:dyDescent="0.35">
@@ -12327,7 +12327,7 @@
         <v>5</v>
       </c>
       <c r="C737" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="738" spans="1:3" x14ac:dyDescent="0.35">
@@ -12536,7 +12536,7 @@
         <v>5</v>
       </c>
       <c r="C756" s="1" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="757" spans="1:3" x14ac:dyDescent="0.35">
@@ -12668,7 +12668,7 @@
         <v>5</v>
       </c>
       <c r="C768" s="1" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="769" spans="1:3" x14ac:dyDescent="0.35">
@@ -12844,7 +12844,7 @@
         <v>2</v>
       </c>
       <c r="C784" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="785" spans="1:3" x14ac:dyDescent="0.35">
@@ -12855,7 +12855,7 @@
         <v>5</v>
       </c>
       <c r="C785" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="786" spans="1:3" x14ac:dyDescent="0.35">
@@ -12910,7 +12910,7 @@
         <v>2</v>
       </c>
       <c r="C790" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="791" spans="1:3" x14ac:dyDescent="0.35">
@@ -12921,7 +12921,7 @@
         <v>5</v>
       </c>
       <c r="C791" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="792" spans="1:3" x14ac:dyDescent="0.35">
@@ -12998,7 +12998,7 @@
         <v>2</v>
       </c>
       <c r="C798" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="799" spans="1:3" x14ac:dyDescent="0.35">
@@ -13009,7 +13009,7 @@
         <v>5</v>
       </c>
       <c r="C799" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="800" spans="1:3" x14ac:dyDescent="0.35">
@@ -13053,7 +13053,7 @@
         <v>1</v>
       </c>
       <c r="C803" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="804" spans="1:3" x14ac:dyDescent="0.35">
@@ -13064,7 +13064,7 @@
         <v>5</v>
       </c>
       <c r="C804" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="805" spans="1:3" x14ac:dyDescent="0.35">
@@ -13075,7 +13075,7 @@
         <v>1</v>
       </c>
       <c r="C805" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="806" spans="1:3" x14ac:dyDescent="0.35">
@@ -13141,7 +13141,7 @@
         <v>2</v>
       </c>
       <c r="C811" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="812" spans="1:3" x14ac:dyDescent="0.35">
@@ -13152,7 +13152,7 @@
         <v>5</v>
       </c>
       <c r="C812" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="813" spans="1:3" x14ac:dyDescent="0.35">
@@ -13559,7 +13559,7 @@
         <v>2</v>
       </c>
       <c r="C849" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="850" spans="1:3" x14ac:dyDescent="0.35">
@@ -13900,7 +13900,7 @@
         <v>1</v>
       </c>
       <c r="C880" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="881" spans="1:3" x14ac:dyDescent="0.35">
@@ -13911,7 +13911,7 @@
         <v>2</v>
       </c>
       <c r="C881" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="882" spans="1:3" x14ac:dyDescent="0.35">
@@ -13999,7 +13999,7 @@
         <v>1</v>
       </c>
       <c r="C889" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="890" spans="1:3" x14ac:dyDescent="0.35">
@@ -14010,7 +14010,7 @@
         <v>2</v>
       </c>
       <c r="C890" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="891" spans="1:3" x14ac:dyDescent="0.35">
@@ -14076,7 +14076,7 @@
         <v>5</v>
       </c>
       <c r="C896" s="1" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="897" spans="1:3" x14ac:dyDescent="0.35">
@@ -14098,7 +14098,7 @@
         <v>1</v>
       </c>
       <c r="C898" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="899" spans="1:3" x14ac:dyDescent="0.35">
@@ -14395,7 +14395,7 @@
         <v>5</v>
       </c>
       <c r="C925" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="926" spans="1:3" x14ac:dyDescent="0.35">
@@ -14472,7 +14472,7 @@
         <v>5</v>
       </c>
       <c r="C932" s="1" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="933" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
modified:   data/chapter2/FRED/subsets/species.xlsx 	modified:   notebooks/chapter_02/paper-draft.ipynb
</commit_message>
<xml_diff>
--- a/data/chapter2/FRED/subsets/species.xlsx
+++ b/data/chapter2/FRED/subsets/species.xlsx
@@ -12676,27 +12676,6 @@
   </cellStyles>
   <dxfs count="18">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
       <font>
         <color rgb="FF9C0006"/>
       </font>
@@ -12725,6 +12704,27 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -12860,13 +12860,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{276A84AE-031F-465C-BBF2-AAF93653128C}" name="species_hand_cleaned" displayName="species_hand_cleaned" ref="A1:G1302" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:G1302" xr:uid="{276A84AE-031F-465C-BBF2-AAF93653128C}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{834DA843-A3B2-4812-B21B-A3DEA02361A7}" uniqueName="1" name="binominal" queryTableFieldId="1" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{25E4C45B-B5E0-47D3-B8D2-D8A032C0B3C1}" uniqueName="2" name="F01286" queryTableFieldId="2" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{BE447818-EF6B-414C-96F1-DF58F4E460AA}" uniqueName="3" name="F01287" queryTableFieldId="3" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{66A0A3E8-604C-477F-BD1E-E7B99F2F3D39}" uniqueName="4" name="F01289" queryTableFieldId="4" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{54B8910C-E82C-4055-9898-875B6ED067C7}" uniqueName="5" name="F01290" queryTableFieldId="5" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{97F66733-E6F6-40AB-B471-ECB89590C4B1}" uniqueName="6" name="reconciled_state" queryTableFieldId="6" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{5BF75914-BDC7-4132-BD06-A237BAE412CF}" uniqueName="7" name="synonyms" queryTableFieldId="7" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{834DA843-A3B2-4812-B21B-A3DEA02361A7}" uniqueName="1" name="binominal" queryTableFieldId="1" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{25E4C45B-B5E0-47D3-B8D2-D8A032C0B3C1}" uniqueName="2" name="F01286" queryTableFieldId="2" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{BE447818-EF6B-414C-96F1-DF58F4E460AA}" uniqueName="3" name="F01287" queryTableFieldId="3" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{66A0A3E8-604C-477F-BD1E-E7B99F2F3D39}" uniqueName="4" name="F01289" queryTableFieldId="4" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{54B8910C-E82C-4055-9898-875B6ED067C7}" uniqueName="5" name="F01290" queryTableFieldId="5" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{97F66733-E6F6-40AB-B471-ECB89590C4B1}" uniqueName="6" name="reconciled_state" queryTableFieldId="6" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{5BF75914-BDC7-4132-BD06-A237BAE412CF}" uniqueName="7" name="synonyms" queryTableFieldId="7" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -23495,7 +23495,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="9" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -24902,7 +24902,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -25482,7 +25482,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
modified:   data/chapter2/FRED/subsets/species.xlsx 	modified:   data/chapter2/FRED/subsets/states.txt
</commit_message>
<xml_diff>
--- a/data/chapter2/FRED/subsets/species.xlsx
+++ b/data/chapter2/FRED/subsets/species.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90963425_westernsydney_edu_au/Documents/PhD/code/data/chapter2/FRED/subsets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="373" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7E43905-9004-4E81-BE57-AEFB2CEE7D6C}"/>
+  <xr:revisionPtr revIDLastSave="376" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{494AE9CA-6E97-4A38-8AAB-644A928A797B}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{A5444074-DC77-415C-A9E2-2BBA8270EAFC}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15125" uniqueCount="4036">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15166" uniqueCount="4036">
   <si>
     <t>F00645</t>
   </si>
@@ -29711,9 +29711,11 @@
         <v>1083</v>
       </c>
       <c r="H137" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I137" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I137" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J137" s="1" t="s">
         <v>1390</v>
       </c>
@@ -29861,9 +29863,11 @@
         <v>1083</v>
       </c>
       <c r="H142" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I142" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I142" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J142" s="1" t="s">
         <v>1083</v>
       </c>
@@ -29951,9 +29955,11 @@
         <v>1083</v>
       </c>
       <c r="H145" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I145" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I145" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J145" s="1" t="s">
         <v>1701</v>
       </c>
@@ -30011,9 +30017,11 @@
         <v>1083</v>
       </c>
       <c r="H147" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I147" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I147" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J147" s="1" t="s">
         <v>1083</v>
       </c>
@@ -30041,9 +30049,11 @@
         <v>1083</v>
       </c>
       <c r="H148" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I148" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I148" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J148" s="1" t="s">
         <v>1916</v>
       </c>
@@ -30491,9 +30501,11 @@
         <v>1083</v>
       </c>
       <c r="H163" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I163" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I163" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J163" s="1" t="s">
         <v>1919</v>
       </c>
@@ -30521,9 +30533,11 @@
         <v>1083</v>
       </c>
       <c r="H164" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I164" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I164" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J164" s="1" t="s">
         <v>1083</v>
       </c>
@@ -30581,9 +30595,11 @@
         <v>1083</v>
       </c>
       <c r="H166" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I166" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I166" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J166" s="1" t="s">
         <v>2142</v>
       </c>
@@ -31151,9 +31167,11 @@
         <v>1083</v>
       </c>
       <c r="H185" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I185" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I185" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J185" s="1" t="s">
         <v>2145</v>
       </c>
@@ -31391,9 +31409,11 @@
         <v>1083</v>
       </c>
       <c r="H193" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I193" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I193" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J193" s="1" t="s">
         <v>1083</v>
       </c>
@@ -31421,9 +31441,11 @@
         <v>1083</v>
       </c>
       <c r="H194" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I194" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I194" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J194" s="1" t="s">
         <v>2418</v>
       </c>
@@ -31631,9 +31653,11 @@
         <v>1083</v>
       </c>
       <c r="H201" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I201" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I201" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J201" s="1" t="s">
         <v>1083</v>
       </c>
@@ -31961,9 +31985,11 @@
         <v>1083</v>
       </c>
       <c r="H212" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I212" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I212" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J212" s="1" t="s">
         <v>1083</v>
       </c>
@@ -32171,9 +32197,11 @@
         <v>1083</v>
       </c>
       <c r="H219" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I219" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I219" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J219" s="1" t="s">
         <v>1083</v>
       </c>
@@ -32231,9 +32259,11 @@
         <v>1083</v>
       </c>
       <c r="H221" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I221" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I221" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J221" s="1" t="s">
         <v>1083</v>
       </c>
@@ -32471,9 +32501,11 @@
         <v>1083</v>
       </c>
       <c r="H229" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I229" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I229" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J229" s="1" t="s">
         <v>2434</v>
       </c>
@@ -32501,9 +32533,11 @@
         <v>1083</v>
       </c>
       <c r="H230" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I230" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I230" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J230" s="1" t="s">
         <v>2438</v>
       </c>
@@ -32651,9 +32685,11 @@
         <v>1083</v>
       </c>
       <c r="H235" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I235" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I235" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J235" s="1" t="s">
         <v>1083</v>
       </c>
@@ -32681,9 +32717,11 @@
         <v>1083</v>
       </c>
       <c r="H236" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I236" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I236" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J236" s="1" t="s">
         <v>1083</v>
       </c>
@@ -32711,9 +32749,11 @@
         <v>1083</v>
       </c>
       <c r="H237" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I237" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I237" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J237" s="1" t="s">
         <v>1083</v>
       </c>
@@ -32741,9 +32781,11 @@
         <v>1083</v>
       </c>
       <c r="H238" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I238" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I238" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J238" s="1" t="s">
         <v>2452</v>
       </c>
@@ -32891,9 +32933,11 @@
         <v>1083</v>
       </c>
       <c r="H243" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I243" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I243" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J243" s="1" t="s">
         <v>2455</v>
       </c>
@@ -33131,9 +33175,11 @@
         <v>1083</v>
       </c>
       <c r="H251" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I251" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I251" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J251" s="1" t="s">
         <v>2458</v>
       </c>
@@ -33521,9 +33567,11 @@
         <v>1083</v>
       </c>
       <c r="H264" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I264" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I264" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J264" s="1" t="s">
         <v>1083</v>
       </c>
@@ -33701,9 +33749,11 @@
         <v>1083</v>
       </c>
       <c r="H270" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I270" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I270" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J270" s="1" t="s">
         <v>1083</v>
       </c>
@@ -33731,9 +33781,11 @@
         <v>1083</v>
       </c>
       <c r="H271" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I271" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I271" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J271" s="1" t="s">
         <v>1083</v>
       </c>
@@ -33821,9 +33873,11 @@
         <v>1083</v>
       </c>
       <c r="H274" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I274" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I274" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J274" s="1" t="s">
         <v>2670</v>
       </c>
@@ -33911,9 +33965,11 @@
         <v>1083</v>
       </c>
       <c r="H277" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I277" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I277" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J277" s="1" t="s">
         <v>3217</v>
       </c>
@@ -34031,9 +34087,11 @@
         <v>1083</v>
       </c>
       <c r="H281" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I281" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I281" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J281" s="1" t="s">
         <v>3737</v>
       </c>
@@ -34061,9 +34119,11 @@
         <v>1083</v>
       </c>
       <c r="H282" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I282" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I282" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J282" s="1" t="s">
         <v>3798</v>
       </c>
@@ -34121,9 +34181,11 @@
         <v>1083</v>
       </c>
       <c r="H284" s="1" t="s">
-        <v>1083</v>
-      </c>
-      <c r="I284" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="I284" s="1" t="s">
+        <v>4035</v>
+      </c>
       <c r="J284" s="1" t="s">
         <v>3808</v>
       </c>

</xml_diff>

<commit_message>
modified:   data/chapter2/FRED/subsets/species.txt 	modified:   data/chapter2/FRED/subsets/species.xlsx 	modified:   notebooks/chapter_02/Wang & Qiu 2006.ipynb
</commit_message>
<xml_diff>
--- a/data/chapter2/FRED/subsets/species.xlsx
+++ b/data/chapter2/FRED/subsets/species.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90963425_westernsydney_edu_au/Documents/PhD/code/data/chapter2/FRED/subsets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="402" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71C13D13-BED1-40C9-BDC8-65CA0F89DD89}"/>
+  <xr:revisionPtr revIDLastSave="415" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F852F72D-3A1E-491E-929D-3CEF7E85B524}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{A5444074-DC77-415C-A9E2-2BBA8270EAFC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="456" activeTab="3" xr2:uid="{A5444074-DC77-415C-A9E2-2BBA8270EAFC}"/>
   </bookViews>
   <sheets>
     <sheet name="FRED4" sheetId="8" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13864" uniqueCount="2975">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13907" uniqueCount="2975">
   <si>
     <t>F00645</t>
   </si>
@@ -35121,9 +35121,11 @@
         <v>1075</v>
       </c>
       <c r="G467" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H467" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H467" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I467" s="1" t="s">
         <v>1075</v>
       </c>
@@ -35175,9 +35177,11 @@
         <v>1075</v>
       </c>
       <c r="G469" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H469" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H469" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I469" s="1" t="s">
         <v>1311</v>
       </c>
@@ -35499,9 +35503,11 @@
         <v>1075</v>
       </c>
       <c r="G481" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H481" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H481" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I481" s="1" t="s">
         <v>1314</v>
       </c>
@@ -35661,9 +35667,11 @@
         <v>1075</v>
       </c>
       <c r="G487" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H487" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H487" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I487" s="1" t="s">
         <v>1393</v>
       </c>
@@ -35688,9 +35696,11 @@
         <v>1075</v>
       </c>
       <c r="G488" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H488" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H488" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I488" s="1" t="s">
         <v>1583</v>
       </c>
@@ -35742,9 +35752,11 @@
         <v>1075</v>
       </c>
       <c r="G490" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H490" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H490" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I490" s="1" t="s">
         <v>1585</v>
       </c>
@@ -35769,9 +35781,11 @@
         <v>1075</v>
       </c>
       <c r="G491" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H491" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H491" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I491" s="1" t="s">
         <v>1632</v>
       </c>
@@ -36338,9 +36352,11 @@
         <v>1075</v>
       </c>
       <c r="G512" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H512" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="H512" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I512" s="1" t="s">
         <v>1075</v>
       </c>
@@ -36392,9 +36408,11 @@
         <v>1075</v>
       </c>
       <c r="G514" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H514" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="H514" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I514" s="1" t="s">
         <v>1441</v>
       </c>
@@ -36419,9 +36437,11 @@
         <v>1075</v>
       </c>
       <c r="G515" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H515" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="H515" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I515" s="1" t="s">
         <v>1075</v>
       </c>
@@ -36446,9 +36466,11 @@
         <v>1075</v>
       </c>
       <c r="G516" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H516" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="H516" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I516" s="1" t="s">
         <v>2141</v>
       </c>
@@ -36473,9 +36495,11 @@
         <v>1075</v>
       </c>
       <c r="G517" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H517" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="H517" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I517" s="1" t="s">
         <v>2145</v>
       </c>
@@ -36662,9 +36686,11 @@
         <v>1075</v>
       </c>
       <c r="G524" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H524" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="H524" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I524" s="1" t="s">
         <v>2148</v>
       </c>
@@ -36743,9 +36769,11 @@
         <v>1075</v>
       </c>
       <c r="G527" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H527" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="H527" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I527" s="1" t="s">
         <v>2151</v>
       </c>
@@ -40772,9 +40800,11 @@
         <v>1075</v>
       </c>
       <c r="G674" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H674" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H674" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I674" s="1" t="s">
         <v>1220</v>
       </c>
@@ -40853,9 +40883,11 @@
         <v>1075</v>
       </c>
       <c r="G677" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H677" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H677" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I677" s="1" t="s">
         <v>1075</v>
       </c>
@@ -41231,9 +41263,11 @@
         <v>1075</v>
       </c>
       <c r="G691" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H691" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H691" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I691" s="1" t="s">
         <v>1075</v>
       </c>
@@ -41258,9 +41292,11 @@
         <v>1075</v>
       </c>
       <c r="G692" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H692" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H692" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I692" s="1" t="s">
         <v>1075</v>
       </c>
@@ -41366,9 +41402,11 @@
         <v>1075</v>
       </c>
       <c r="G696" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H696" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H696" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I696" s="1" t="s">
         <v>1075</v>
       </c>
@@ -41501,9 +41539,11 @@
         <v>1075</v>
       </c>
       <c r="G701" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H701" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H701" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I701" s="1" t="s">
         <v>2254</v>
       </c>
@@ -41555,9 +41595,11 @@
         <v>1075</v>
       </c>
       <c r="G703" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H703" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H703" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I703" s="1" t="s">
         <v>1075</v>
       </c>
@@ -41636,9 +41678,11 @@
         <v>1075</v>
       </c>
       <c r="G706" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H706" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H706" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I706" s="1" t="s">
         <v>2257</v>
       </c>
@@ -41798,9 +41842,11 @@
         <v>1075</v>
       </c>
       <c r="G712" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H712" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H712" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I712" s="1" t="s">
         <v>1075</v>
       </c>
@@ -41825,9 +41871,11 @@
         <v>1075</v>
       </c>
       <c r="G713" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H713" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H713" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I713" s="1" t="s">
         <v>2260</v>
       </c>
@@ -41933,9 +41981,11 @@
         <v>1075</v>
       </c>
       <c r="G717" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H717" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H717" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I717" s="1" t="s">
         <v>2262</v>
       </c>
@@ -42149,9 +42199,11 @@
         <v>1075</v>
       </c>
       <c r="G725" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H725" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H725" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I725" s="1" t="s">
         <v>2521</v>
       </c>

</xml_diff>

<commit_message>
modified:   data/chapter2/FRED/subsets/species.txt 	modified:   data/chapter2/FRED/subsets/species.xlsx
</commit_message>
<xml_diff>
--- a/data/chapter2/FRED/subsets/species.xlsx
+++ b/data/chapter2/FRED/subsets/species.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90963425_westernsydney_edu_au/Documents/PhD/code/data/chapter2/FRED/subsets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="415" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F852F72D-3A1E-491E-929D-3CEF7E85B524}"/>
+  <xr:revisionPtr revIDLastSave="424" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4A5B090-3767-43C1-ADD4-90828592DC7B}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="456" activeTab="3" xr2:uid="{A5444074-DC77-415C-A9E2-2BBA8270EAFC}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13907" uniqueCount="2975">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13945" uniqueCount="2975">
   <si>
     <t>F00645</t>
   </si>
@@ -42417,9 +42417,11 @@
         <v>1075</v>
       </c>
       <c r="G733" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H733" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H733" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I733" s="1" t="s">
         <v>1137</v>
       </c>
@@ -43443,9 +43445,11 @@
         <v>1075</v>
       </c>
       <c r="G771" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H771" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H771" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I771" s="1" t="s">
         <v>1075</v>
       </c>
@@ -43470,9 +43474,11 @@
         <v>1075</v>
       </c>
       <c r="G772" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H772" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H772" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I772" s="1" t="s">
         <v>1460</v>
       </c>
@@ -43740,9 +43746,11 @@
         <v>1075</v>
       </c>
       <c r="G782" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H782" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H782" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I782" s="1" t="s">
         <v>1075</v>
       </c>
@@ -43956,9 +43964,11 @@
         <v>1075</v>
       </c>
       <c r="G790" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H790" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H790" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I790" s="1" t="s">
         <v>1075</v>
       </c>
@@ -43983,9 +43993,11 @@
         <v>1075</v>
       </c>
       <c r="G791" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H791" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H791" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I791" s="1" t="s">
         <v>2671</v>
       </c>
@@ -44010,9 +44022,11 @@
         <v>1075</v>
       </c>
       <c r="G792" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H792" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H792" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I792" s="1" t="s">
         <v>1075</v>
       </c>
@@ -44037,9 +44051,11 @@
         <v>1075</v>
       </c>
       <c r="G793" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H793" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H793" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I793" s="1" t="s">
         <v>1075</v>
       </c>
@@ -44064,9 +44080,11 @@
         <v>1075</v>
       </c>
       <c r="G794" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H794" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H794" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I794" s="1" t="s">
         <v>1075</v>
       </c>
@@ -44091,9 +44109,11 @@
         <v>1075</v>
       </c>
       <c r="G795" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H795" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H795" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I795" s="1" t="s">
         <v>1075</v>
       </c>
@@ -44172,9 +44192,11 @@
         <v>1075</v>
       </c>
       <c r="G798" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H798" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H798" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I798" s="1" t="s">
         <v>1075</v>
       </c>
@@ -44442,9 +44464,11 @@
         <v>1075</v>
       </c>
       <c r="G808" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H808" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H808" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I808" s="1" t="s">
         <v>1817</v>
       </c>
@@ -44496,9 +44520,11 @@
         <v>1075</v>
       </c>
       <c r="G810" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H810" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H810" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I810" s="1" t="s">
         <v>1075</v>
       </c>
@@ -44523,9 +44549,11 @@
         <v>1075</v>
       </c>
       <c r="G811" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H811" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H811" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I811" s="1" t="s">
         <v>1075</v>
       </c>
@@ -44550,9 +44578,11 @@
         <v>1075</v>
       </c>
       <c r="G812" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H812" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H812" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I812" s="1" t="s">
         <v>1075</v>
       </c>
@@ -44577,9 +44607,11 @@
         <v>1075</v>
       </c>
       <c r="G813" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H813" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H813" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I813" s="1" t="s">
         <v>1075</v>
       </c>
@@ -45036,9 +45068,11 @@
         <v>1075</v>
       </c>
       <c r="G830" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H830" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H830" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I830" s="1" t="s">
         <v>1964</v>
       </c>
@@ -45117,9 +45151,11 @@
         <v>1075</v>
       </c>
       <c r="G833" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H833" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H833" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I833" s="1" t="s">
         <v>1075</v>
       </c>
@@ -45144,9 +45180,11 @@
         <v>1075</v>
       </c>
       <c r="G834" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H834" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H834" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I834" s="1" t="s">
         <v>1075</v>
       </c>
@@ -45171,9 +45209,11 @@
         <v>1075</v>
       </c>
       <c r="G835" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H835" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H835" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I835" s="1" t="s">
         <v>2598</v>
       </c>
@@ -45819,9 +45859,11 @@
         <v>1075</v>
       </c>
       <c r="G859" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H859" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H859" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I859" s="1" t="s">
         <v>1075</v>
       </c>
@@ -45954,9 +45996,11 @@
         <v>1075</v>
       </c>
       <c r="G864" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H864" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H864" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I864" s="1" t="s">
         <v>1788</v>
       </c>
@@ -46062,9 +46106,11 @@
         <v>1075</v>
       </c>
       <c r="G868" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H868" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H868" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I868" s="1" t="s">
         <v>2305</v>
       </c>
@@ -50868,9 +50914,11 @@
         <v>1075</v>
       </c>
       <c r="G1046" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1046" s="1"/>
+        <v>5</v>
+      </c>
+      <c r="H1046" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I1046" s="1" t="s">
         <v>1075</v>
       </c>
@@ -50976,9 +51024,11 @@
         <v>1075</v>
       </c>
       <c r="G1050" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1050" s="1"/>
+        <v>5</v>
+      </c>
+      <c r="H1050" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I1050" s="1" t="s">
         <v>1075</v>
       </c>
@@ -51084,9 +51134,11 @@
         <v>1075</v>
       </c>
       <c r="G1054" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1054" s="1"/>
+        <v>5</v>
+      </c>
+      <c r="H1054" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I1054" s="1" t="s">
         <v>1075</v>
       </c>
@@ -51381,9 +51433,11 @@
         <v>1075</v>
       </c>
       <c r="G1065" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1065" s="1"/>
+        <v>5</v>
+      </c>
+      <c r="H1065" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I1065" s="1" t="s">
         <v>1075</v>
       </c>
@@ -52150,9 +52204,11 @@
         <v>1075</v>
       </c>
       <c r="G1092" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1092" s="1"/>
+        <v>5</v>
+      </c>
+      <c r="H1092" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I1092" s="1" t="s">
         <v>1075</v>
       </c>

</xml_diff>

<commit_message>
modified:   R/notebooks/MRPMM.ipynb 	modified:   data/chapter2/FRED/subsets/species.changelog 	modified:   data/chapter2/FRED/subsets/species.xlsx
</commit_message>
<xml_diff>
--- a/data/chapter2/FRED/subsets/species.xlsx
+++ b/data/chapter2/FRED/subsets/species.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90963425_westernsydney_edu_au/Documents/PhD/code/data/chapter2/FRED/subsets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="446" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD15912E-3F11-480A-ACCE-D32D195EEC2D}"/>
+  <xr:revisionPtr revIDLastSave="468" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BA45933-51B2-4564-A2E2-006DD58694A2}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="456" activeTab="3" xr2:uid="{A5444074-DC77-415C-A9E2-2BBA8270EAFC}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13983" uniqueCount="2975">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14031" uniqueCount="2975">
   <si>
     <t>F00645</t>
   </si>
@@ -25440,7 +25440,7 @@
         <v>1277</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>2386</v>
       </c>
@@ -25604,7 +25604,7 @@
         <v>1284</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
         <v>2727</v>
       </c>
@@ -26038,7 +26038,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
         <v>1351</v>
       </c>
@@ -26058,14 +26058,16 @@
         <v>1075</v>
       </c>
       <c r="G134" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H134" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H134" s="1" t="s">
+        <v>2969</v>
+      </c>
       <c r="I134" s="1" t="s">
         <v>1075</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>1353</v>
       </c>
@@ -26085,9 +26087,11 @@
         <v>1075</v>
       </c>
       <c r="G135" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H135" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H135" s="1" t="s">
+        <v>2969</v>
+      </c>
       <c r="I135" s="1" t="s">
         <v>1075</v>
       </c>
@@ -30177,7 +30181,7 @@
         <v>2810</v>
       </c>
     </row>
-    <row r="285" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A285" s="1" t="s">
         <v>1641</v>
       </c>
@@ -30206,7 +30210,7 @@
         <v>1643</v>
       </c>
     </row>
-    <row r="286" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A286" s="1" t="s">
         <v>1845</v>
       </c>
@@ -30559,7 +30563,7 @@
         <v>1568</v>
       </c>
     </row>
-    <row r="299" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A299" s="1" t="s">
         <v>2881</v>
       </c>
@@ -30804,7 +30808,7 @@
         <v>1580</v>
       </c>
     </row>
-    <row r="308" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A308" s="1" t="s">
         <v>1467</v>
       </c>
@@ -30824,14 +30828,16 @@
         <v>1075</v>
       </c>
       <c r="G308" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H308" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H308" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I308" s="1" t="s">
         <v>1075</v>
       </c>
     </row>
-    <row r="309" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A309" s="1" t="s">
         <v>2799</v>
       </c>
@@ -30851,9 +30857,11 @@
         <v>1075</v>
       </c>
       <c r="G309" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H309" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H309" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I309" s="1" t="s">
         <v>2801</v>
       </c>
@@ -31209,7 +31217,7 @@
         <v>1605</v>
       </c>
     </row>
-    <row r="323" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A323" s="1" t="s">
         <v>1888</v>
       </c>
@@ -31229,14 +31237,16 @@
         <v>1075</v>
       </c>
       <c r="G323" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H323" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H323" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I323" s="1" t="s">
         <v>1890</v>
       </c>
     </row>
-    <row r="324" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A324" s="1" t="s">
         <v>1502</v>
       </c>
@@ -31256,9 +31266,11 @@
         <v>1075</v>
       </c>
       <c r="G324" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H324" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H324" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I324" s="1" t="s">
         <v>1075</v>
       </c>
@@ -31290,7 +31302,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="326" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A326" s="1" t="s">
         <v>1918</v>
       </c>
@@ -31310,14 +31322,16 @@
         <v>1075</v>
       </c>
       <c r="G326" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H326" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H326" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I326" s="1" t="s">
         <v>1920</v>
       </c>
     </row>
-    <row r="327" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A327" s="1" t="s">
         <v>1921</v>
       </c>
@@ -31337,9 +31351,11 @@
         <v>1075</v>
       </c>
       <c r="G327" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H327" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H327" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I327" s="1" t="s">
         <v>1075</v>
       </c>
@@ -31587,7 +31603,7 @@
         <v>1625</v>
       </c>
     </row>
-    <row r="337" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A337" s="1" t="s">
         <v>2115</v>
       </c>
@@ -31607,14 +31623,16 @@
         <v>1075</v>
       </c>
       <c r="G337" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H337" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H337" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I337" s="1" t="s">
         <v>1075</v>
       </c>
     </row>
-    <row r="338" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A338" s="1" t="s">
         <v>2116</v>
       </c>
@@ -31634,9 +31652,11 @@
         <v>1075</v>
       </c>
       <c r="G338" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H338" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H338" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I338" s="1" t="s">
         <v>1075</v>
       </c>
@@ -31803,7 +31823,7 @@
         <v>1640</v>
       </c>
     </row>
-    <row r="345" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A345" s="1" t="s">
         <v>2117</v>
       </c>
@@ -31823,9 +31843,11 @@
         <v>1075</v>
       </c>
       <c r="G345" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H345" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H345" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I345" s="1" t="s">
         <v>1075</v>
       </c>
@@ -32596,7 +32618,7 @@
         <v>1927</v>
       </c>
     </row>
-    <row r="374" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A374" s="1" t="s">
         <v>1539</v>
       </c>
@@ -32616,9 +32638,11 @@
         <v>1075</v>
       </c>
       <c r="G374" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H374" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H374" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I374" s="1" t="s">
         <v>1542</v>
       </c>
@@ -32866,7 +32890,7 @@
         <v>1720</v>
       </c>
     </row>
-    <row r="384" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A384" s="1" t="s">
         <v>1548</v>
       </c>
@@ -32886,9 +32910,11 @@
         <v>1075</v>
       </c>
       <c r="G384" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H384" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H384" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I384" s="1" t="s">
         <v>1075</v>
       </c>
@@ -33163,7 +33189,7 @@
         <v>1732</v>
       </c>
     </row>
-    <row r="395" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A395" s="1" t="s">
         <v>1551</v>
       </c>
@@ -33183,14 +33209,16 @@
         <v>1075</v>
       </c>
       <c r="G395" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H395" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H395" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I395" s="1" t="s">
         <v>1075</v>
       </c>
     </row>
-    <row r="396" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="396" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A396" s="1" t="s">
         <v>1552</v>
       </c>
@@ -33210,9 +33238,11 @@
         <v>1075</v>
       </c>
       <c r="G396" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H396" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H396" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I396" s="1" t="s">
         <v>1075</v>
       </c>
@@ -33578,7 +33608,7 @@
         <v>2948</v>
       </c>
     </row>
-    <row r="410" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="410" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A410" s="1" t="s">
         <v>1408</v>
       </c>
@@ -33598,9 +33628,11 @@
         <v>1075</v>
       </c>
       <c r="G410" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H410" s="1"/>
+        <v>4</v>
+      </c>
+      <c r="H410" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I410" s="1" t="s">
         <v>1411</v>
       </c>
@@ -33632,7 +33664,7 @@
         <v>1763</v>
       </c>
     </row>
-    <row r="412" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="412" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A412" s="1" t="s">
         <v>1412</v>
       </c>
@@ -33652,14 +33684,16 @@
         <v>1075</v>
       </c>
       <c r="G412" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H412" s="1"/>
+        <v>4</v>
+      </c>
+      <c r="H412" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I412" s="1" t="s">
         <v>1413</v>
       </c>
     </row>
-    <row r="413" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="413" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A413" s="1" t="s">
         <v>1417</v>
       </c>
@@ -33679,9 +33713,11 @@
         <v>1075</v>
       </c>
       <c r="G413" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H413" s="1"/>
+        <v>4</v>
+      </c>
+      <c r="H413" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I413" s="1" t="s">
         <v>1418</v>
       </c>
@@ -56724,7 +56760,7 @@
         <v>2896</v>
       </c>
     </row>
-    <row r="1258" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1258" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1258" s="1" t="s">
         <v>1484</v>
       </c>
@@ -56744,9 +56780,11 @@
         <v>1075</v>
       </c>
       <c r="G1258" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1258" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1258" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I1258" s="1" t="s">
         <v>1075</v>
       </c>
@@ -56940,7 +56978,7 @@
         <v>2906</v>
       </c>
     </row>
-    <row r="1266" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1266" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1266" s="1" t="s">
         <v>2469</v>
       </c>
@@ -56960,9 +56998,11 @@
         <v>1075</v>
       </c>
       <c r="G1266" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1266" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1266" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I1266" s="1" t="s">
         <v>1075</v>
       </c>
@@ -57021,7 +57061,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="1269" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1269" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1269" s="1" t="s">
         <v>2950</v>
       </c>
@@ -57041,9 +57081,11 @@
         <v>1075</v>
       </c>
       <c r="G1269" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1269" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1269" s="1" t="s">
+        <v>2974</v>
+      </c>
       <c r="I1269" s="1" t="s">
         <v>2952</v>
       </c>

</xml_diff>

<commit_message>
modified:   R/notebooks/MRPMM.ipynb 	modified:   data/chapter2/FRED/subsets/species.xlsx
</commit_message>
<xml_diff>
--- a/data/chapter2/FRED/subsets/species.xlsx
+++ b/data/chapter2/FRED/subsets/species.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90963425_westernsydney_edu_au/Documents/PhD/code/data/chapter2/FRED/subsets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="468" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BA45933-51B2-4564-A2E2-006DD58694A2}"/>
+  <xr:revisionPtr revIDLastSave="526" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D97DE75E-1679-42F4-9C00-D4BEAF07C48B}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="456" activeTab="3" xr2:uid="{A5444074-DC77-415C-A9E2-2BBA8270EAFC}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14031" uniqueCount="2975">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14087" uniqueCount="2977">
   <si>
     <t>F00645</t>
   </si>
@@ -8986,14 +8986,43 @@
     <t>Luke</t>
   </si>
   <si>
-    <t>Brundrett &amp; Tedersoo 2018</t>
+    <r>
+      <t xml:space="preserve">(Soudzilovskaia </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>et al.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, 2020)</t>
+    </r>
+  </si>
+  <si>
+    <t>(Soudzilovskaia et al., 2020)</t>
+  </si>
+  <si>
+    <t>(Brundrett and Tedersoo, 2018)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -9130,6 +9159,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -9723,6 +9760,9 @@
     <filterColumn colId="6">
       <filters blank="1"/>
     </filterColumn>
+    <filterColumn colId="7">
+      <filters blank="1"/>
+    </filterColumn>
   </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A38:I1294">
     <sortCondition ref="C2:C1302"/>
@@ -22373,7 +22413,7 @@
     <col min="4" max="4" width="26.453125" customWidth="1"/>
     <col min="5" max="5" width="17.08984375" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="17.26953125" customWidth="1"/>
-    <col min="8" max="8" width="23" customWidth="1"/>
+    <col min="8" max="8" width="26.54296875" customWidth="1"/>
     <col min="9" max="9" width="89.54296875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -23437,7 +23477,7 @@
         <v>2</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I38" s="1" t="s">
         <v>1075</v>
@@ -23547,7 +23587,7 @@
         <v>2</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I42" s="1" t="s">
         <v>2132</v>
@@ -23576,7 +23616,7 @@
         <v>2</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I43" s="1" t="s">
         <v>2134</v>
@@ -23767,7 +23807,7 @@
         <v>2</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I50" s="1" t="s">
         <v>1075</v>
@@ -23796,7 +23836,7 @@
         <v>2</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I51" s="1" t="s">
         <v>1075</v>
@@ -24095,7 +24135,7 @@
         <v>2</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I62" s="1" t="s">
         <v>1075</v>
@@ -24259,7 +24299,7 @@
         <v>2</v>
       </c>
       <c r="H68" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I68" s="1" t="s">
         <v>2280</v>
@@ -24531,7 +24571,7 @@
         <v>2</v>
       </c>
       <c r="H78" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I78" s="1" t="s">
         <v>2284</v>
@@ -24560,7 +24600,7 @@
         <v>2</v>
       </c>
       <c r="H79" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I79" s="1" t="s">
         <v>2909</v>
@@ -24616,7 +24656,7 @@
         <v>2</v>
       </c>
       <c r="H81" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I81" s="1" t="s">
         <v>2291</v>
@@ -24645,7 +24685,7 @@
         <v>2</v>
       </c>
       <c r="H82" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I82" s="1" t="s">
         <v>2868</v>
@@ -24674,7 +24714,7 @@
         <v>2</v>
       </c>
       <c r="H83" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I83" s="1" t="s">
         <v>1075</v>
@@ -24757,7 +24797,7 @@
         <v>2</v>
       </c>
       <c r="H86" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I86" s="1" t="s">
         <v>2010</v>
@@ -25056,7 +25096,7 @@
         <v>2</v>
       </c>
       <c r="H97" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I97" s="1" t="s">
         <v>1075</v>
@@ -25463,7 +25503,7 @@
         <v>2</v>
       </c>
       <c r="H112" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I112" s="1" t="s">
         <v>2388</v>
@@ -25627,7 +25667,7 @@
         <v>2</v>
       </c>
       <c r="H118" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I118" s="1" t="s">
         <v>2729</v>
@@ -26061,7 +26101,7 @@
         <v>2</v>
       </c>
       <c r="H134" s="1" t="s">
-        <v>2969</v>
+        <v>2975</v>
       </c>
       <c r="I134" s="1" t="s">
         <v>1075</v>
@@ -26090,7 +26130,7 @@
         <v>2</v>
       </c>
       <c r="H135" s="1" t="s">
-        <v>2969</v>
+        <v>2975</v>
       </c>
       <c r="I135" s="1" t="s">
         <v>1075</v>
@@ -26146,7 +26186,7 @@
         <v>2</v>
       </c>
       <c r="H137" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I137" s="1" t="s">
         <v>1280</v>
@@ -26283,7 +26323,7 @@
         <v>2</v>
       </c>
       <c r="H142" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I142" s="1" t="s">
         <v>1075</v>
@@ -26366,7 +26406,7 @@
         <v>2</v>
       </c>
       <c r="H145" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I145" s="1" t="s">
         <v>1473</v>
@@ -26422,7 +26462,7 @@
         <v>2</v>
       </c>
       <c r="H147" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I147" s="1" t="s">
         <v>1075</v>
@@ -26451,7 +26491,7 @@
         <v>2</v>
       </c>
       <c r="H148" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I148" s="1" t="s">
         <v>1608</v>
@@ -26858,7 +26898,7 @@
         <v>2</v>
       </c>
       <c r="H163" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I163" s="1" t="s">
         <v>1610</v>
@@ -26887,7 +26927,7 @@
         <v>2</v>
       </c>
       <c r="H164" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I164" s="1" t="s">
         <v>1075</v>
@@ -26943,7 +26983,7 @@
         <v>2</v>
       </c>
       <c r="H166" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I166" s="1" t="s">
         <v>1759</v>
@@ -27458,7 +27498,7 @@
         <v>2</v>
       </c>
       <c r="H185" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I185" s="1" t="s">
         <v>1761</v>
@@ -27676,7 +27716,7 @@
         <v>2</v>
       </c>
       <c r="H193" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I193" s="1" t="s">
         <v>1075</v>
@@ -27705,7 +27745,7 @@
         <v>2</v>
       </c>
       <c r="H194" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I194" s="1" t="s">
         <v>1931</v>
@@ -27896,7 +27936,7 @@
         <v>2</v>
       </c>
       <c r="H201" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I201" s="1" t="s">
         <v>1075</v>
@@ -28195,7 +28235,7 @@
         <v>2</v>
       </c>
       <c r="H212" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I212" s="1" t="s">
         <v>1075</v>
@@ -28386,7 +28426,7 @@
         <v>2</v>
       </c>
       <c r="H219" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I219" s="1" t="s">
         <v>1075</v>
@@ -28442,7 +28482,7 @@
         <v>2</v>
       </c>
       <c r="H221" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I221" s="1" t="s">
         <v>1075</v>
@@ -28660,7 +28700,7 @@
         <v>2</v>
       </c>
       <c r="H229" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I229" s="1" t="s">
         <v>1939</v>
@@ -28689,7 +28729,7 @@
         <v>2</v>
       </c>
       <c r="H230" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I230" s="1" t="s">
         <v>1941</v>
@@ -28826,7 +28866,7 @@
         <v>2</v>
       </c>
       <c r="H235" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I235" s="1" t="s">
         <v>1075</v>
@@ -28855,7 +28895,7 @@
         <v>2</v>
       </c>
       <c r="H236" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I236" s="1" t="s">
         <v>1075</v>
@@ -28884,7 +28924,7 @@
         <v>2</v>
       </c>
       <c r="H237" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I237" s="1" t="s">
         <v>1075</v>
@@ -28913,7 +28953,7 @@
         <v>2</v>
       </c>
       <c r="H238" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I238" s="1" t="s">
         <v>1948</v>
@@ -29050,7 +29090,7 @@
         <v>2</v>
       </c>
       <c r="H243" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I243" s="1" t="s">
         <v>1950</v>
@@ -29268,7 +29308,7 @@
         <v>2</v>
       </c>
       <c r="H251" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I251" s="1" t="s">
         <v>1952</v>
@@ -29621,7 +29661,7 @@
         <v>2</v>
       </c>
       <c r="H264" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I264" s="1" t="s">
         <v>1075</v>
@@ -29785,7 +29825,7 @@
         <v>2</v>
       </c>
       <c r="H270" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I270" s="1" t="s">
         <v>1075</v>
@@ -29814,7 +29854,7 @@
         <v>2</v>
       </c>
       <c r="H271" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I271" s="1" t="s">
         <v>1075</v>
@@ -29897,7 +29937,7 @@
         <v>2</v>
       </c>
       <c r="H274" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I274" s="1" t="s">
         <v>2082</v>
@@ -29980,7 +30020,7 @@
         <v>2</v>
       </c>
       <c r="H277" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I277" s="1" t="s">
         <v>2423</v>
@@ -30090,7 +30130,7 @@
         <v>2</v>
       </c>
       <c r="H281" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I281" s="1" t="s">
         <v>2761</v>
@@ -30119,7 +30159,7 @@
         <v>2</v>
       </c>
       <c r="H282" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I282" s="1" t="s">
         <v>2804</v>
@@ -30175,7 +30215,7 @@
         <v>2</v>
       </c>
       <c r="H284" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I284" s="1" t="s">
         <v>2810</v>
@@ -30204,7 +30244,7 @@
         <v>2</v>
       </c>
       <c r="H285" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I285" s="1" t="s">
         <v>1643</v>
@@ -30233,7 +30273,7 @@
         <v>2</v>
       </c>
       <c r="H286" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I286" s="1" t="s">
         <v>1847</v>
@@ -30586,7 +30626,7 @@
         <v>2</v>
       </c>
       <c r="H299" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I299" s="1" t="s">
         <v>1075</v>
@@ -30831,7 +30871,7 @@
         <v>2</v>
       </c>
       <c r="H308" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I308" s="1" t="s">
         <v>1075</v>
@@ -30860,7 +30900,7 @@
         <v>2</v>
       </c>
       <c r="H309" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I309" s="1" t="s">
         <v>2801</v>
@@ -31240,7 +31280,7 @@
         <v>2</v>
       </c>
       <c r="H323" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I323" s="1" t="s">
         <v>1890</v>
@@ -31269,7 +31309,7 @@
         <v>2</v>
       </c>
       <c r="H324" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I324" s="1" t="s">
         <v>1075</v>
@@ -31325,7 +31365,7 @@
         <v>2</v>
       </c>
       <c r="H326" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I326" s="1" t="s">
         <v>1920</v>
@@ -31354,7 +31394,7 @@
         <v>2</v>
       </c>
       <c r="H327" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I327" s="1" t="s">
         <v>1075</v>
@@ -31626,7 +31666,7 @@
         <v>2</v>
       </c>
       <c r="H337" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I337" s="1" t="s">
         <v>1075</v>
@@ -31655,7 +31695,7 @@
         <v>2</v>
       </c>
       <c r="H338" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I338" s="1" t="s">
         <v>1075</v>
@@ -31846,7 +31886,7 @@
         <v>2</v>
       </c>
       <c r="H345" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I345" s="1" t="s">
         <v>1075</v>
@@ -31929,7 +31969,7 @@
         <v>1</v>
       </c>
       <c r="H348" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I348" s="1" t="s">
         <v>1527</v>
@@ -32120,7 +32160,7 @@
         <v>1</v>
       </c>
       <c r="H355" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I355" s="1" t="s">
         <v>1529</v>
@@ -32446,7 +32486,7 @@
         <v>1</v>
       </c>
       <c r="H367" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I367" s="1" t="s">
         <v>1075</v>
@@ -32529,7 +32569,7 @@
         <v>1</v>
       </c>
       <c r="H370" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I370" s="1" t="s">
         <v>1925</v>
@@ -32612,7 +32652,7 @@
         <v>1</v>
       </c>
       <c r="H373" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I373" s="1" t="s">
         <v>1927</v>
@@ -32641,7 +32681,7 @@
         <v>2</v>
       </c>
       <c r="H374" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I374" s="1" t="s">
         <v>1542</v>
@@ -32913,7 +32953,7 @@
         <v>2</v>
       </c>
       <c r="H384" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I384" s="1" t="s">
         <v>1075</v>
@@ -33212,7 +33252,7 @@
         <v>2</v>
       </c>
       <c r="H395" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I395" s="1" t="s">
         <v>1075</v>
@@ -33241,7 +33281,7 @@
         <v>2</v>
       </c>
       <c r="H396" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I396" s="1" t="s">
         <v>1075</v>
@@ -33324,7 +33364,7 @@
         <v>2</v>
       </c>
       <c r="H399" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I399" s="1" t="s">
         <v>2942</v>
@@ -33353,7 +33393,7 @@
         <v>2</v>
       </c>
       <c r="H400" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I400" s="1" t="s">
         <v>2944</v>
@@ -33409,7 +33449,7 @@
         <v>2</v>
       </c>
       <c r="H402" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I402" s="1" t="s">
         <v>1075</v>
@@ -33546,7 +33586,7 @@
         <v>2</v>
       </c>
       <c r="H407" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I407" s="1" t="s">
         <v>1075</v>
@@ -33602,7 +33642,7 @@
         <v>2</v>
       </c>
       <c r="H409" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I409" s="1" t="s">
         <v>2948</v>
@@ -33631,7 +33671,7 @@
         <v>4</v>
       </c>
       <c r="H410" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I410" s="1" t="s">
         <v>1411</v>
@@ -33687,7 +33727,7 @@
         <v>4</v>
       </c>
       <c r="H412" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I412" s="1" t="s">
         <v>1413</v>
@@ -33716,7 +33756,7 @@
         <v>4</v>
       </c>
       <c r="H413" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I413" s="1" t="s">
         <v>1418</v>
@@ -34147,9 +34187,11 @@
         <v>1075</v>
       </c>
       <c r="G429" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H429" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H429" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="I429" s="1" t="s">
         <v>1629</v>
       </c>
@@ -34336,9 +34378,11 @@
         <v>1075</v>
       </c>
       <c r="G436" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H436" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="H436" s="1" t="s">
+        <v>2976</v>
+      </c>
       <c r="I436" s="1" t="s">
         <v>2662</v>
       </c>
@@ -34498,9 +34542,11 @@
         <v>1075</v>
       </c>
       <c r="G442" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H442" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="H442" s="1" t="s">
+        <v>2976</v>
+      </c>
       <c r="I442" s="1" t="s">
         <v>2676</v>
       </c>
@@ -34660,9 +34706,11 @@
         <v>1075</v>
       </c>
       <c r="G448" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H448" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H448" s="1" t="s">
+        <v>2976</v>
+      </c>
       <c r="I448" s="1" t="s">
         <v>1075</v>
       </c>
@@ -34822,9 +34870,11 @@
         <v>1075</v>
       </c>
       <c r="G454" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H454" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H454" s="1" t="s">
+        <v>2976</v>
+      </c>
       <c r="I454" s="1" t="s">
         <v>1075</v>
       </c>
@@ -34929,10 +34979,12 @@
       <c r="F458" s="1" t="s">
         <v>1075</v>
       </c>
-      <c r="G458" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H458" s="1"/>
+      <c r="G458" t="s">
+        <v>2</v>
+      </c>
+      <c r="H458" t="s">
+        <v>2975</v>
+      </c>
       <c r="I458" s="1" t="s">
         <v>1075</v>
       </c>
@@ -35065,9 +35117,11 @@
         <v>1075</v>
       </c>
       <c r="G463" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H463" s="1"/>
+        <v>6</v>
+      </c>
+      <c r="H463" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="I463" s="1" t="s">
         <v>1755</v>
       </c>
@@ -35176,7 +35230,7 @@
         <v>2</v>
       </c>
       <c r="H467" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I467" s="1" t="s">
         <v>1075</v>
@@ -35232,7 +35286,7 @@
         <v>2</v>
       </c>
       <c r="H469" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I469" s="1" t="s">
         <v>1311</v>
@@ -35558,7 +35612,7 @@
         <v>2</v>
       </c>
       <c r="H481" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I481" s="1" t="s">
         <v>1314</v>
@@ -35722,7 +35776,7 @@
         <v>2</v>
       </c>
       <c r="H487" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I487" s="1" t="s">
         <v>1393</v>
@@ -35751,7 +35805,7 @@
         <v>2</v>
       </c>
       <c r="H488" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I488" s="1" t="s">
         <v>1583</v>
@@ -35807,7 +35861,7 @@
         <v>2</v>
       </c>
       <c r="H490" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I490" s="1" t="s">
         <v>1585</v>
@@ -35836,7 +35890,7 @@
         <v>2</v>
       </c>
       <c r="H491" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I491" s="1" t="s">
         <v>1632</v>
@@ -36324,7 +36378,7 @@
         <v>5</v>
       </c>
       <c r="H509" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I509" s="1" t="s">
         <v>1075</v>
@@ -36407,7 +36461,7 @@
         <v>1</v>
       </c>
       <c r="H512" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I512" s="1" t="s">
         <v>1075</v>
@@ -36463,7 +36517,7 @@
         <v>1</v>
       </c>
       <c r="H514" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I514" s="1" t="s">
         <v>1441</v>
@@ -36492,7 +36546,7 @@
         <v>1</v>
       </c>
       <c r="H515" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I515" s="1" t="s">
         <v>1075</v>
@@ -36521,7 +36575,7 @@
         <v>1</v>
       </c>
       <c r="H516" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I516" s="1" t="s">
         <v>2141</v>
@@ -36550,7 +36604,7 @@
         <v>1</v>
       </c>
       <c r="H517" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I517" s="1" t="s">
         <v>2145</v>
@@ -36741,7 +36795,7 @@
         <v>1</v>
       </c>
       <c r="H524" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I524" s="1" t="s">
         <v>2148</v>
@@ -36824,7 +36878,7 @@
         <v>1</v>
       </c>
       <c r="H527" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I527" s="1" t="s">
         <v>2151</v>
@@ -37015,7 +37069,7 @@
         <v>2</v>
       </c>
       <c r="H534" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I534" s="1" t="s">
         <v>1129</v>
@@ -37098,7 +37152,7 @@
         <v>2</v>
       </c>
       <c r="H537" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I537" s="1" t="s">
         <v>1545</v>
@@ -37127,7 +37181,7 @@
         <v>2</v>
       </c>
       <c r="H538" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I538" s="1" t="s">
         <v>1914</v>
@@ -37156,7 +37210,7 @@
         <v>2</v>
       </c>
       <c r="H539" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I539" s="1" t="s">
         <v>2591</v>
@@ -37212,7 +37266,7 @@
         <v>2</v>
       </c>
       <c r="H541" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I541" s="1" t="s">
         <v>2742</v>
@@ -37241,7 +37295,7 @@
         <v>2</v>
       </c>
       <c r="H542" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I542" s="1" t="s">
         <v>1075</v>
@@ -37297,7 +37351,7 @@
         <v>2</v>
       </c>
       <c r="H544" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I544" s="1" t="s">
         <v>1075</v>
@@ -37326,7 +37380,7 @@
         <v>2</v>
       </c>
       <c r="H545" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I545" s="1" t="s">
         <v>1159</v>
@@ -37409,7 +37463,7 @@
         <v>2</v>
       </c>
       <c r="H548" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I548" s="1" t="s">
         <v>1197</v>
@@ -37465,7 +37519,7 @@
         <v>2</v>
       </c>
       <c r="H550" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I550" s="1" t="s">
         <v>1230</v>
@@ -37548,7 +37602,7 @@
         <v>2</v>
       </c>
       <c r="H553" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I553" s="1" t="s">
         <v>1234</v>
@@ -37577,7 +37631,7 @@
         <v>2</v>
       </c>
       <c r="H554" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I554" s="1" t="s">
         <v>1075</v>
@@ -37606,7 +37660,7 @@
         <v>2</v>
       </c>
       <c r="H555" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I555" s="1" t="s">
         <v>1075</v>
@@ -37635,7 +37689,7 @@
         <v>2</v>
       </c>
       <c r="H556" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I556" s="1" t="s">
         <v>1075</v>
@@ -37664,7 +37718,7 @@
         <v>2</v>
       </c>
       <c r="H557" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I557" s="1" t="s">
         <v>1075</v>
@@ -37693,7 +37747,7 @@
         <v>2</v>
       </c>
       <c r="H558" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I558" s="1" t="s">
         <v>1075</v>
@@ -37857,7 +37911,7 @@
         <v>2</v>
       </c>
       <c r="H564" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I564" s="1" t="s">
         <v>1075</v>
@@ -38048,7 +38102,7 @@
         <v>2</v>
       </c>
       <c r="H571" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I571" s="1" t="s">
         <v>2157</v>
@@ -38077,7 +38131,7 @@
         <v>2</v>
       </c>
       <c r="H572" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I572" s="1" t="s">
         <v>1075</v>
@@ -38106,7 +38160,7 @@
         <v>2</v>
       </c>
       <c r="H573" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I573" s="1" t="s">
         <v>2163</v>
@@ -38135,7 +38189,7 @@
         <v>2</v>
       </c>
       <c r="H574" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I574" s="1" t="s">
         <v>2184</v>
@@ -38164,7 +38218,7 @@
         <v>2</v>
       </c>
       <c r="H575" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I575" s="1" t="s">
         <v>1075</v>
@@ -38274,7 +38328,7 @@
         <v>2</v>
       </c>
       <c r="H579" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I579" s="1" t="s">
         <v>2368</v>
@@ -38492,7 +38546,7 @@
         <v>2</v>
       </c>
       <c r="H587" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I587" s="1" t="s">
         <v>1075</v>
@@ -38521,7 +38575,7 @@
         <v>2</v>
       </c>
       <c r="H588" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I588" s="1" t="s">
         <v>1075</v>
@@ -38550,7 +38604,7 @@
         <v>2</v>
       </c>
       <c r="H589" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I589" s="1" t="s">
         <v>1075</v>
@@ -38633,7 +38687,7 @@
         <v>2</v>
       </c>
       <c r="H592" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I592" s="1" t="s">
         <v>1075</v>
@@ -38878,7 +38932,7 @@
         <v>2</v>
       </c>
       <c r="H601" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I601" s="1" t="s">
         <v>2446</v>
@@ -38988,7 +39042,7 @@
         <v>2</v>
       </c>
       <c r="H605" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I605" s="1" t="s">
         <v>1075</v>
@@ -39152,7 +39206,7 @@
         <v>2</v>
       </c>
       <c r="H611" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I611" s="1" t="s">
         <v>1075</v>
@@ -40855,7 +40909,7 @@
         <v>2</v>
       </c>
       <c r="H674" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I674" s="1" t="s">
         <v>1220</v>
@@ -40938,7 +40992,7 @@
         <v>2</v>
       </c>
       <c r="H677" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I677" s="1" t="s">
         <v>1075</v>
@@ -41318,7 +41372,7 @@
         <v>2</v>
       </c>
       <c r="H691" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I691" s="1" t="s">
         <v>1075</v>
@@ -41347,7 +41401,7 @@
         <v>2</v>
       </c>
       <c r="H692" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I692" s="1" t="s">
         <v>1075</v>
@@ -41457,7 +41511,7 @@
         <v>2</v>
       </c>
       <c r="H696" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I696" s="1" t="s">
         <v>1075</v>
@@ -41594,7 +41648,7 @@
         <v>2</v>
       </c>
       <c r="H701" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I701" s="1" t="s">
         <v>2254</v>
@@ -41650,7 +41704,7 @@
         <v>2</v>
       </c>
       <c r="H703" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I703" s="1" t="s">
         <v>1075</v>
@@ -41733,7 +41787,7 @@
         <v>2</v>
       </c>
       <c r="H706" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I706" s="1" t="s">
         <v>2257</v>
@@ -41897,7 +41951,7 @@
         <v>2</v>
       </c>
       <c r="H712" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I712" s="1" t="s">
         <v>1075</v>
@@ -41926,7 +41980,7 @@
         <v>2</v>
       </c>
       <c r="H713" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I713" s="1" t="s">
         <v>2260</v>
@@ -42036,7 +42090,7 @@
         <v>2</v>
       </c>
       <c r="H717" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I717" s="1" t="s">
         <v>2262</v>
@@ -42254,7 +42308,7 @@
         <v>2</v>
       </c>
       <c r="H725" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I725" s="1" t="s">
         <v>2521</v>
@@ -42472,7 +42526,7 @@
         <v>2</v>
       </c>
       <c r="H733" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I733" s="1" t="s">
         <v>1137</v>
@@ -43500,7 +43554,7 @@
         <v>2</v>
       </c>
       <c r="H771" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I771" s="1" t="s">
         <v>1075</v>
@@ -43529,7 +43583,7 @@
         <v>2</v>
       </c>
       <c r="H772" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I772" s="1" t="s">
         <v>1460</v>
@@ -43801,7 +43855,7 @@
         <v>2</v>
       </c>
       <c r="H782" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I782" s="1" t="s">
         <v>1075</v>
@@ -44019,7 +44073,7 @@
         <v>2</v>
       </c>
       <c r="H790" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I790" s="1" t="s">
         <v>1075</v>
@@ -44048,7 +44102,7 @@
         <v>2</v>
       </c>
       <c r="H791" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I791" s="1" t="s">
         <v>2671</v>
@@ -44077,7 +44131,7 @@
         <v>2</v>
       </c>
       <c r="H792" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I792" s="1" t="s">
         <v>1075</v>
@@ -44106,7 +44160,7 @@
         <v>2</v>
       </c>
       <c r="H793" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I793" s="1" t="s">
         <v>1075</v>
@@ -44135,7 +44189,7 @@
         <v>2</v>
       </c>
       <c r="H794" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I794" s="1" t="s">
         <v>1075</v>
@@ -44164,7 +44218,7 @@
         <v>2</v>
       </c>
       <c r="H795" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I795" s="1" t="s">
         <v>1075</v>
@@ -44247,7 +44301,7 @@
         <v>2</v>
       </c>
       <c r="H798" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I798" s="1" t="s">
         <v>1075</v>
@@ -44519,7 +44573,7 @@
         <v>2</v>
       </c>
       <c r="H808" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I808" s="1" t="s">
         <v>1817</v>
@@ -44575,7 +44629,7 @@
         <v>2</v>
       </c>
       <c r="H810" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I810" s="1" t="s">
         <v>1075</v>
@@ -44604,7 +44658,7 @@
         <v>2</v>
       </c>
       <c r="H811" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I811" s="1" t="s">
         <v>1075</v>
@@ -44633,7 +44687,7 @@
         <v>2</v>
       </c>
       <c r="H812" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I812" s="1" t="s">
         <v>1075</v>
@@ -44662,7 +44716,7 @@
         <v>2</v>
       </c>
       <c r="H813" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I813" s="1" t="s">
         <v>1075</v>
@@ -45123,7 +45177,7 @@
         <v>2</v>
       </c>
       <c r="H830" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I830" s="1" t="s">
         <v>1964</v>
@@ -45206,7 +45260,7 @@
         <v>2</v>
       </c>
       <c r="H833" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I833" s="1" t="s">
         <v>1075</v>
@@ -45235,7 +45289,7 @@
         <v>2</v>
       </c>
       <c r="H834" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I834" s="1" t="s">
         <v>1075</v>
@@ -45264,7 +45318,7 @@
         <v>2</v>
       </c>
       <c r="H835" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I835" s="1" t="s">
         <v>2598</v>
@@ -45914,7 +45968,7 @@
         <v>2</v>
       </c>
       <c r="H859" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I859" s="1" t="s">
         <v>1075</v>
@@ -46051,7 +46105,7 @@
         <v>2</v>
       </c>
       <c r="H864" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I864" s="1" t="s">
         <v>1788</v>
@@ -46161,7 +46215,7 @@
         <v>2</v>
       </c>
       <c r="H868" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I868" s="1" t="s">
         <v>2305</v>
@@ -48188,7 +48242,7 @@
         <v>2</v>
       </c>
       <c r="H943" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I943" s="1" t="s">
         <v>1470</v>
@@ -48325,7 +48379,7 @@
         <v>2</v>
       </c>
       <c r="H948" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I948" s="1" t="s">
         <v>1650</v>
@@ -48354,7 +48408,7 @@
         <v>2</v>
       </c>
       <c r="H949" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I949" s="1" t="s">
         <v>1722</v>
@@ -48788,7 +48842,7 @@
         <v>2</v>
       </c>
       <c r="H965" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I965" s="1" t="s">
         <v>1075</v>
@@ -48979,7 +49033,7 @@
         <v>2</v>
       </c>
       <c r="H972" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I972" s="1" t="s">
         <v>1075</v>
@@ -49035,7 +49089,7 @@
         <v>2</v>
       </c>
       <c r="H974" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I974" s="1" t="s">
         <v>2518</v>
@@ -49172,7 +49226,7 @@
         <v>2</v>
       </c>
       <c r="H979" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I979" s="1" t="s">
         <v>2620</v>
@@ -49201,7 +49255,7 @@
         <v>2</v>
       </c>
       <c r="H980" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I980" s="1" t="s">
         <v>2782</v>
@@ -50985,7 +51039,7 @@
         <v>5</v>
       </c>
       <c r="H1046" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1046" s="1" t="s">
         <v>1075</v>
@@ -51095,7 +51149,7 @@
         <v>5</v>
       </c>
       <c r="H1050" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1050" s="1" t="s">
         <v>1075</v>
@@ -51205,7 +51259,7 @@
         <v>5</v>
       </c>
       <c r="H1054" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1054" s="1" t="s">
         <v>1075</v>
@@ -51504,7 +51558,7 @@
         <v>5</v>
       </c>
       <c r="H1065" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1065" s="1" t="s">
         <v>1075</v>
@@ -52275,7 +52329,7 @@
         <v>5</v>
       </c>
       <c r="H1092" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1092" s="1" t="s">
         <v>1075</v>
@@ -52713,7 +52767,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="1109" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1109" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1109" s="1" t="s">
         <v>1699</v>
       </c>
@@ -52733,14 +52787,16 @@
         <v>1075</v>
       </c>
       <c r="G1109" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1109" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1109" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="I1109" s="1" t="s">
         <v>1701</v>
       </c>
     </row>
-    <row r="1110" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1110" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1110" s="1" t="s">
         <v>2583</v>
       </c>
@@ -52760,9 +52816,11 @@
         <v>1075</v>
       </c>
       <c r="G1110" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1110" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1110" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="I1110" s="1" t="s">
         <v>1075</v>
       </c>
@@ -52794,7 +52852,7 @@
         <v>2673</v>
       </c>
     </row>
-    <row r="1112" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1112" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1112" s="1" t="s">
         <v>2584</v>
       </c>
@@ -52814,9 +52872,11 @@
         <v>1075</v>
       </c>
       <c r="G1112" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1112" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1112" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="I1112" s="1" t="s">
         <v>2585</v>
       </c>
@@ -53118,7 +53178,7 @@
         <v>2687</v>
       </c>
     </row>
-    <row r="1124" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1124" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1124" s="1" t="s">
         <v>2664</v>
       </c>
@@ -53138,9 +53198,11 @@
         <v>1075</v>
       </c>
       <c r="G1124" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1124" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1124" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="I1124" s="1" t="s">
         <v>2665</v>
       </c>
@@ -53388,7 +53450,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="1134" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1134" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1134" s="1" t="s">
         <v>2768</v>
       </c>
@@ -53408,9 +53470,11 @@
         <v>1075</v>
       </c>
       <c r="G1134" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1134" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1134" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="I1134" s="1" t="s">
         <v>2769</v>
       </c>
@@ -53519,7 +53583,7 @@
         <v>2</v>
       </c>
       <c r="H1138" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1138" s="1" t="s">
         <v>1331</v>
@@ -53791,7 +53855,7 @@
         <v>2</v>
       </c>
       <c r="H1148" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1148" s="1" t="s">
         <v>1075</v>
@@ -53847,7 +53911,7 @@
         <v>2</v>
       </c>
       <c r="H1150" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1150" s="1" t="s">
         <v>2004</v>
@@ -53957,7 +54021,7 @@
         <v>2</v>
       </c>
       <c r="H1154" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1154" s="1" t="s">
         <v>2072</v>
@@ -54013,7 +54077,7 @@
         <v>2</v>
       </c>
       <c r="H1156" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1156" s="1" t="s">
         <v>1075</v>
@@ -54042,7 +54106,7 @@
         <v>2</v>
       </c>
       <c r="H1157" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1157" s="1" t="s">
         <v>2414</v>
@@ -54071,7 +54135,7 @@
         <v>2</v>
       </c>
       <c r="H1158" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1158" s="1" t="s">
         <v>2416</v>
@@ -54100,7 +54164,7 @@
         <v>2</v>
       </c>
       <c r="H1159" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1159" s="1" t="s">
         <v>2268</v>
@@ -54264,7 +54328,7 @@
         <v>2</v>
       </c>
       <c r="H1165" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1165" s="1" t="s">
         <v>2914</v>
@@ -54648,7 +54712,7 @@
         <v>2780</v>
       </c>
     </row>
-    <row r="1180" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1180" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1180" s="1" t="s">
         <v>2688</v>
       </c>
@@ -54668,9 +54732,11 @@
         <v>1075</v>
       </c>
       <c r="G1180" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1180" s="1"/>
+        <v>3</v>
+      </c>
+      <c r="H1180" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="I1180" s="1" t="s">
         <v>1075</v>
       </c>
@@ -54725,7 +54791,7 @@
         <v>2</v>
       </c>
       <c r="H1182" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1182" s="1" t="s">
         <v>1181</v>
@@ -54970,7 +55036,7 @@
         <v>2</v>
       </c>
       <c r="H1191" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1191" s="1" t="s">
         <v>1075</v>
@@ -54999,7 +55065,7 @@
         <v>2</v>
       </c>
       <c r="H1192" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1192" s="1" t="s">
         <v>1075</v>
@@ -55113,7 +55179,7 @@
         <v>2808</v>
       </c>
     </row>
-    <row r="1197" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1197" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1197" s="1" t="s">
         <v>2503</v>
       </c>
@@ -55133,9 +55199,11 @@
         <v>1075</v>
       </c>
       <c r="G1197" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1197" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1197" s="1" t="s">
+        <v>2976</v>
+      </c>
       <c r="I1197" s="1" t="s">
         <v>2505</v>
       </c>
@@ -55842,7 +55910,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="1224" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1224" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1224" s="1" t="s">
         <v>2549</v>
       </c>
@@ -55862,9 +55930,11 @@
         <v>1075</v>
       </c>
       <c r="G1224" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1224" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1224" s="1" t="s">
+        <v>2976</v>
+      </c>
       <c r="I1224" s="1" t="s">
         <v>2551</v>
       </c>
@@ -56274,7 +56344,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="1240" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1240" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1240" s="1" t="s">
         <v>1154</v>
       </c>
@@ -56294,9 +56364,11 @@
         <v>1075</v>
       </c>
       <c r="G1240" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1240" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1240" s="1" t="s">
+        <v>2976</v>
+      </c>
       <c r="I1240" s="1" t="s">
         <v>1075</v>
       </c>
@@ -56382,7 +56454,7 @@
         <v>2873</v>
       </c>
     </row>
-    <row r="1244" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1244" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1244" s="1" t="s">
         <v>2478</v>
       </c>
@@ -56402,9 +56474,11 @@
         <v>1075</v>
       </c>
       <c r="G1244" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1244" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1244" s="1" t="s">
+        <v>2976</v>
+      </c>
       <c r="I1244" s="1" t="s">
         <v>1075</v>
       </c>
@@ -56463,7 +56537,7 @@
         <v>2880</v>
       </c>
     </row>
-    <row r="1247" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1247" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1247" s="1" t="s">
         <v>2745</v>
       </c>
@@ -56483,14 +56557,16 @@
         <v>1075</v>
       </c>
       <c r="G1247" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1247" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1247" s="1" t="s">
+        <v>2976</v>
+      </c>
       <c r="I1247" s="1" t="s">
         <v>2748</v>
       </c>
     </row>
-    <row r="1248" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1248" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1248" s="1" t="s">
         <v>2749</v>
       </c>
@@ -56510,9 +56586,11 @@
         <v>1075</v>
       </c>
       <c r="G1248" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1248" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1248" s="1" t="s">
+        <v>2976</v>
+      </c>
       <c r="I1248" s="1" t="s">
         <v>2750</v>
       </c>
@@ -56783,7 +56861,7 @@
         <v>2</v>
       </c>
       <c r="H1258" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1258" s="1" t="s">
         <v>1075</v>
@@ -57001,7 +57079,7 @@
         <v>2</v>
       </c>
       <c r="H1266" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1266" s="1" t="s">
         <v>1075</v>
@@ -57084,7 +57162,7 @@
         <v>2</v>
       </c>
       <c r="H1269" s="1" t="s">
-        <v>2974</v>
+        <v>2976</v>
       </c>
       <c r="I1269" s="1" t="s">
         <v>2952</v>
@@ -57252,7 +57330,7 @@
         <v>2925</v>
       </c>
     </row>
-    <row r="1276" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1276" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1276" s="1" t="s">
         <v>2897</v>
       </c>
@@ -57272,9 +57350,11 @@
         <v>1075</v>
       </c>
       <c r="G1276" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1276" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1276" s="1" t="s">
+        <v>2976</v>
+      </c>
       <c r="I1276" s="1" t="s">
         <v>2901</v>
       </c>
@@ -57306,7 +57386,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="1278" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1278" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1278" s="1" t="s">
         <v>1900</v>
       </c>
@@ -57326,9 +57406,11 @@
         <v>1075</v>
       </c>
       <c r="G1278" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1278" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1278" s="1" t="s">
+        <v>2976</v>
+      </c>
       <c r="I1278" s="1" t="s">
         <v>1075</v>
       </c>
@@ -57549,7 +57631,7 @@
         <v>2939</v>
       </c>
     </row>
-    <row r="1287" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1287" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1287" s="1" t="s">
         <v>1874</v>
       </c>
@@ -57569,14 +57651,16 @@
         <v>1075</v>
       </c>
       <c r="G1287" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1287" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1287" s="1" t="s">
+        <v>2976</v>
+      </c>
       <c r="I1287" s="1" t="s">
         <v>1877</v>
       </c>
     </row>
-    <row r="1288" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1288" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1288" s="1" t="s">
         <v>1455</v>
       </c>
@@ -57596,9 +57680,11 @@
         <v>1075</v>
       </c>
       <c r="G1288" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1288" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1288" t="s">
+        <v>2974</v>
+      </c>
       <c r="I1288" s="1" t="s">
         <v>1075</v>
       </c>
@@ -57630,7 +57716,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="1290" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1290" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1290" s="1" t="s">
         <v>2547</v>
       </c>
@@ -57650,14 +57736,16 @@
         <v>1075</v>
       </c>
       <c r="G1290" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1290" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1290" t="s">
+        <v>2975</v>
+      </c>
       <c r="I1290" s="1" t="s">
         <v>1075</v>
       </c>
     </row>
-    <row r="1291" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1291" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1291" s="1" t="s">
         <v>2930</v>
       </c>
@@ -57677,9 +57765,11 @@
         <v>1075</v>
       </c>
       <c r="G1291" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1291" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1291" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="I1291" s="1" t="s">
         <v>1075</v>
       </c>
@@ -57738,7 +57828,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="1294" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1294" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1294" s="1" t="s">
         <v>2087</v>
       </c>
@@ -57758,9 +57848,11 @@
         <v>1075</v>
       </c>
       <c r="G1294" s="1" t="s">
-        <v>1075</v>
-      </c>
-      <c r="H1294" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="H1294" s="1" t="s">
+        <v>2976</v>
+      </c>
       <c r="I1294" s="1" t="s">
         <v>2090</v>
       </c>

</xml_diff>

<commit_message>
modified:   data/chapter2/FRED/subsets/species.changelog 	modified:   data/chapter2/FRED/subsets/species.xlsx 	modified:   notebooks/chapter_02/paper-draft.ipynb
</commit_message>
<xml_diff>
--- a/data/chapter2/FRED/subsets/species.xlsx
+++ b/data/chapter2/FRED/subsets/species.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90963425_westernsydney_edu_au/Documents/PhD/code/data/chapter2/FRED/subsets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="667" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5FCA0E6-0A85-4C64-9343-999E046C39CC}"/>
+  <xr:revisionPtr revIDLastSave="684" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC17E4B3-8AE3-4185-9D2F-E2E2FA36B7DC}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="456" activeTab="3" xr2:uid="{A5444074-DC77-415C-A9E2-2BBA8270EAFC}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15359" uniqueCount="2979">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15365" uniqueCount="2979">
   <si>
     <t>F00645</t>
   </si>
@@ -9773,7 +9773,7 @@
   <autoFilter ref="A1:K1302" xr:uid="{92DE4C38-9658-4F81-87D7-16EF2BBFE835}">
     <filterColumn colId="2">
       <filters>
-        <filter val="Cornaceae"/>
+        <filter val="Cyperaceae"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -24068,7 +24068,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>114</v>
       </c>
@@ -28551,7 +28551,7 @@
         <v>1931</v>
       </c>
     </row>
-    <row r="195" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A195" s="1" t="s">
         <v>23</v>
       </c>
@@ -28575,14 +28575,16 @@
       </c>
       <c r="H195" s="1"/>
       <c r="I195" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J195" s="1"/>
+        <v>4</v>
+      </c>
+      <c r="J195" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K195" s="1" t="s">
         <v>1414</v>
       </c>
     </row>
-    <row r="196" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A196" s="1" t="s">
         <v>202</v>
       </c>
@@ -28613,7 +28615,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="197" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A197" s="1" t="s">
         <v>203</v>
       </c>
@@ -28637,14 +28639,16 @@
       </c>
       <c r="H197" s="1"/>
       <c r="I197" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J197" s="1"/>
+        <v>4</v>
+      </c>
+      <c r="J197" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K197" s="1" t="s">
         <v>1075</v>
       </c>
     </row>
-    <row r="198" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A198" s="1" t="s">
         <v>932</v>
       </c>
@@ -28675,7 +28679,7 @@
         <v>1415</v>
       </c>
     </row>
-    <row r="199" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A199" s="1" t="s">
         <v>204</v>
       </c>
@@ -28699,14 +28703,16 @@
       </c>
       <c r="H199" s="1"/>
       <c r="I199" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J199" s="1"/>
+        <v>4</v>
+      </c>
+      <c r="J199" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K199" s="1" t="s">
         <v>1075</v>
       </c>
     </row>
-    <row r="200" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A200" s="1" t="s">
         <v>205</v>
       </c>
@@ -28770,7 +28776,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="202" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A202" s="1" t="s">
         <v>941</v>
       </c>
@@ -31918,7 +31924,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="302" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A302" s="1" t="s">
         <v>269</v>
       </c>
@@ -31949,7 +31955,7 @@
         <v>1575</v>
       </c>
     </row>
-    <row r="303" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A303" s="1" t="s">
         <v>270</v>
       </c>
@@ -31980,7 +31986,7 @@
         <v>1576</v>
       </c>
     </row>
-    <row r="304" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A304" s="1" t="s">
         <v>271</v>
       </c>
@@ -32011,7 +32017,7 @@
         <v>1577</v>
       </c>
     </row>
-    <row r="305" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A305" s="1" t="s">
         <v>272</v>
       </c>
@@ -32042,7 +32048,7 @@
         <v>1578</v>
       </c>
     </row>
-    <row r="306" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A306" s="1" t="s">
         <v>273</v>
       </c>
@@ -32075,7 +32081,7 @@
         <v>1579</v>
       </c>
     </row>
-    <row r="307" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A307" s="1" t="s">
         <v>274</v>
       </c>
@@ -35316,7 +35322,7 @@
         <v>2948</v>
       </c>
     </row>
-    <row r="410" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+    <row r="410" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A410" s="1" t="s">
         <v>1408</v>
       </c>
@@ -35380,7 +35386,7 @@
         <v>1763</v>
       </c>
     </row>
-    <row r="412" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+    <row r="412" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A412" s="1" t="s">
         <v>1412</v>
       </c>
@@ -35413,7 +35419,7 @@
         <v>1413</v>
       </c>
     </row>
-    <row r="413" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+    <row r="413" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A413" s="1" t="s">
         <v>1417</v>
       </c>
@@ -37486,7 +37492,7 @@
         <v>1833</v>
       </c>
     </row>
-    <row r="479" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+    <row r="479" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A479" s="1" t="s">
         <v>392</v>
       </c>
@@ -37510,14 +37516,16 @@
       </c>
       <c r="H479" s="1"/>
       <c r="I479" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="J479" s="1"/>
+        <v>4</v>
+      </c>
+      <c r="J479" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K479" s="1" t="s">
         <v>1075</v>
       </c>
     </row>
-    <row r="480" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+    <row r="480" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A480" s="1" t="s">
         <v>393</v>
       </c>
@@ -37541,9 +37549,11 @@
       </c>
       <c r="H480" s="1"/>
       <c r="I480" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="J480" s="1"/>
+        <v>4</v>
+      </c>
+      <c r="J480" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K480" s="1" t="s">
         <v>1835</v>
       </c>
@@ -42278,9 +42288,11 @@
       </c>
       <c r="H629" s="1"/>
       <c r="I629" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J629" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="J629" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K629" s="1" t="s">
         <v>2047</v>
       </c>

</xml_diff>

<commit_message>
modified:   data/chapter2/Brundrett and Tedersoo 2018 - mycorrhizal associations.xlsx 	modified:   data/chapter2/FRED/subsets/species.xlsx 	modified:   notebooks/chapter_02/paper-draft.ipynb
</commit_message>
<xml_diff>
--- a/data/chapter2/FRED/subsets/species.xlsx
+++ b/data/chapter2/FRED/subsets/species.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90963425_westernsydney_edu_au/Documents/PhD/code/data/chapter2/FRED/subsets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="738" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00D8A1E6-40F6-4111-9A85-996DE538BE4B}"/>
+  <xr:revisionPtr revIDLastSave="813" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87EEBF4A-DAA0-4826-94E6-4564C75A0E5B}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="456" activeTab="3" xr2:uid="{A5444074-DC77-415C-A9E2-2BBA8270EAFC}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15383" uniqueCount="2979">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15411" uniqueCount="2979">
   <si>
     <t>F00645</t>
   </si>
@@ -9771,9 +9771,9 @@
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{92DE4C38-9658-4F81-87D7-16EF2BBFE835}" name="species_hand_cleaned__2" displayName="species_hand_cleaned__2" ref="A1:K1302" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:K1302" xr:uid="{92DE4C38-9658-4F81-87D7-16EF2BBFE835}">
-    <filterColumn colId="2">
+    <filterColumn colId="1">
       <filters>
-        <filter val="Fabaceae"/>
+        <filter val="Oreocnide"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -22531,7 +22531,7 @@
         <v>1064</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>75</v>
       </c>
@@ -22564,7 +22564,7 @@
         <v>1068</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>76</v>
       </c>
@@ -22595,7 +22595,7 @@
         <v>1069</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>77</v>
       </c>
@@ -25265,7 +25265,7 @@
         <v>1236</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>12</v>
       </c>
@@ -25296,7 +25296,7 @@
         <v>1238</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>1045</v>
       </c>
@@ -25351,9 +25351,11 @@
       </c>
       <c r="H92" s="1"/>
       <c r="I92" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J92" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="J92" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K92" s="1" t="s">
         <v>1242</v>
       </c>
@@ -25641,7 +25643,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>144</v>
       </c>
@@ -25672,7 +25674,7 @@
         <v>1260</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>145</v>
       </c>
@@ -25789,9 +25791,11 @@
       </c>
       <c r="H106" s="1"/>
       <c r="I106" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J106" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="J106" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K106" s="1" t="s">
         <v>1264</v>
       </c>
@@ -26705,7 +26709,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>1308</v>
       </c>
@@ -26771,7 +26775,7 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>1310</v>
       </c>
@@ -26961,7 +26965,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
         <v>1006</v>
       </c>
@@ -27432,7 +27436,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
         <v>1313</v>
       </c>
@@ -27929,9 +27933,11 @@
       </c>
       <c r="H174" s="1"/>
       <c r="I174" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J174" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="J174" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K174" s="1" t="s">
         <v>1370</v>
       </c>
@@ -28122,7 +28128,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181" s="1" t="s">
         <v>959</v>
       </c>
@@ -29156,9 +29162,11 @@
       </c>
       <c r="H213" s="1"/>
       <c r="I213" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="J213" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="J213" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K213" s="1" t="s">
         <v>1436</v>
       </c>
@@ -29470,9 +29478,11 @@
       </c>
       <c r="H223" s="1"/>
       <c r="I223" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J223" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="J223" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K223" s="1" t="s">
         <v>1444</v>
       </c>
@@ -30047,7 +30057,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="242" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A242" s="1" t="s">
         <v>19</v>
       </c>
@@ -30111,7 +30121,7 @@
         <v>1950</v>
       </c>
     </row>
-    <row r="244" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A244" s="1" t="s">
         <v>947</v>
       </c>
@@ -31267,9 +31277,11 @@
       </c>
       <c r="H280" s="1"/>
       <c r="I280" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J280" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="J280" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K280" s="1" t="s">
         <v>1538</v>
       </c>
@@ -31340,7 +31352,7 @@
         <v>2804</v>
       </c>
     </row>
-    <row r="283" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A283" s="1" t="s">
         <v>192</v>
       </c>
@@ -31494,9 +31506,11 @@
       </c>
       <c r="H287" s="1"/>
       <c r="I287" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J287" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="J287" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K287" s="1" t="s">
         <v>1075</v>
       </c>
@@ -31525,9 +31539,11 @@
       </c>
       <c r="H288" s="1"/>
       <c r="I288" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J288" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="J288" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K288" s="1" t="s">
         <v>1555</v>
       </c>
@@ -33358,7 +33374,7 @@
         <v>1645</v>
       </c>
     </row>
-    <row r="347" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A347" s="1" t="s">
         <v>1391</v>
       </c>
@@ -33572,9 +33588,11 @@
       </c>
       <c r="H353" s="1"/>
       <c r="I353" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J353" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="J353" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K353" s="1" t="s">
         <v>1663</v>
       </c>
@@ -33791,9 +33809,11 @@
       </c>
       <c r="H360" s="1"/>
       <c r="I360" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J360" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="J360" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K360" s="1" t="s">
         <v>1678</v>
       </c>
@@ -35210,9 +35230,11 @@
       </c>
       <c r="H405" s="1"/>
       <c r="I405" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="J405" s="1"/>
+        <v>4</v>
+      </c>
+      <c r="J405" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K405" s="1" t="s">
         <v>1751</v>
       </c>
@@ -36811,9 +36833,11 @@
       </c>
       <c r="H456" s="1"/>
       <c r="I456" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J456" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="J456" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K456" s="1" t="s">
         <v>1811</v>
       </c>
@@ -36842,9 +36866,11 @@
       </c>
       <c r="H457" s="1"/>
       <c r="I457" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J457" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="J457" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K457" s="1" t="s">
         <v>1812</v>
       </c>
@@ -37137,7 +37163,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="467" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="467" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A467" s="1" t="s">
         <v>231</v>
       </c>
@@ -37199,7 +37225,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="469" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="469" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A469" s="1" t="s">
         <v>951</v>
       </c>
@@ -37577,7 +37603,7 @@
         <v>1835</v>
       </c>
     </row>
-    <row r="481" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="481" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A481" s="1" t="s">
         <v>257</v>
       </c>
@@ -37763,7 +37789,7 @@
         <v>1844</v>
       </c>
     </row>
-    <row r="487" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="487" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A487" s="1" t="s">
         <v>1581</v>
       </c>
@@ -37796,7 +37822,7 @@
         <v>1583</v>
       </c>
     </row>
-    <row r="488" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="488" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A488" s="1" t="s">
         <v>1584</v>
       </c>
@@ -37829,7 +37855,7 @@
         <v>1585</v>
       </c>
     </row>
-    <row r="489" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="489" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A489" s="1" t="s">
         <v>1630</v>
       </c>
@@ -37862,7 +37888,7 @@
         <v>1632</v>
       </c>
     </row>
-    <row r="490" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="490" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A490" s="1" t="s">
         <v>29</v>
       </c>
@@ -37893,7 +37919,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="491" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="491" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A491" s="1" t="s">
         <v>1666</v>
       </c>
@@ -38021,7 +38047,7 @@
         <v>1864</v>
       </c>
     </row>
-    <row r="495" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="495" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A495" s="1" t="s">
         <v>1705</v>
       </c>
@@ -38054,7 +38080,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="496" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="496" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A496" s="1" t="s">
         <v>398</v>
       </c>
@@ -38085,7 +38111,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="497" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="497" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A497" s="1" t="s">
         <v>1851</v>
       </c>
@@ -38182,7 +38208,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="500" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="500" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A500" s="1" t="s">
         <v>401</v>
       </c>
@@ -38237,14 +38263,16 @@
       </c>
       <c r="H501" s="1"/>
       <c r="I501" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J501" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="J501" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K501" s="1" t="s">
         <v>1075</v>
       </c>
     </row>
-    <row r="502" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="502" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A502" s="1" t="s">
         <v>948</v>
       </c>
@@ -38275,7 +38303,7 @@
         <v>2015</v>
       </c>
     </row>
-    <row r="503" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="503" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A503" s="1" t="s">
         <v>425</v>
       </c>
@@ -38306,7 +38334,7 @@
         <v>2017</v>
       </c>
     </row>
-    <row r="504" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="504" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A504" s="1" t="s">
         <v>426</v>
       </c>
@@ -38368,7 +38396,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="506" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="506" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A506" s="1" t="s">
         <v>427</v>
       </c>
@@ -38399,7 +38427,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="507" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="507" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A507" s="1" t="s">
         <v>428</v>
       </c>
@@ -38461,7 +38489,7 @@
         <v>1887</v>
       </c>
     </row>
-    <row r="509" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="509" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A509" s="1" t="s">
         <v>429</v>
       </c>
@@ -38523,7 +38551,7 @@
         <v>1894</v>
       </c>
     </row>
-    <row r="511" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="511" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A511" s="1" t="s">
         <v>430</v>
       </c>
@@ -41176,7 +41204,7 @@
         <v>2013</v>
       </c>
     </row>
-    <row r="594" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="594" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A594" s="1" t="s">
         <v>2020</v>
       </c>
@@ -41209,7 +41237,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="595" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="595" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A595" s="1" t="s">
         <v>431</v>
       </c>
@@ -41240,7 +41268,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="596" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="596" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A596" s="1" t="s">
         <v>432</v>
       </c>
@@ -41271,7 +41299,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="597" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="597" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A597" s="1" t="s">
         <v>433</v>
       </c>
@@ -41302,7 +41330,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="598" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="598" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A598" s="1" t="s">
         <v>2022</v>
       </c>
@@ -41335,7 +41363,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="599" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="599" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A599" s="1" t="s">
         <v>434</v>
       </c>
@@ -41366,7 +41394,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="600" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="600" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A600" s="1" t="s">
         <v>435</v>
       </c>
@@ -41430,7 +41458,7 @@
         <v>2446</v>
       </c>
     </row>
-    <row r="602" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="602" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A602" s="1" t="s">
         <v>45</v>
       </c>
@@ -41461,7 +41489,7 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="603" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="603" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A603" s="1" t="s">
         <v>436</v>
       </c>
@@ -41492,7 +41520,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="604" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="604" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A604" s="1" t="s">
         <v>437</v>
       </c>
@@ -41556,7 +41584,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="606" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="606" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A606" s="1" t="s">
         <v>2026</v>
       </c>
@@ -41589,7 +41617,7 @@
         <v>2027</v>
       </c>
     </row>
-    <row r="607" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="607" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A607" s="1" t="s">
         <v>438</v>
       </c>
@@ -41620,7 +41648,7 @@
         <v>2028</v>
       </c>
     </row>
-    <row r="608" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="608" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A608" s="1" t="s">
         <v>439</v>
       </c>
@@ -41651,7 +41679,7 @@
         <v>2029</v>
       </c>
     </row>
-    <row r="609" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="609" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A609" s="1" t="s">
         <v>440</v>
       </c>
@@ -41682,7 +41710,7 @@
         <v>2030</v>
       </c>
     </row>
-    <row r="610" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="610" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A610" s="1" t="s">
         <v>441</v>
       </c>
@@ -41746,7 +41774,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="612" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="612" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A612" s="1" t="s">
         <v>442</v>
       </c>
@@ -41777,7 +41805,7 @@
         <v>2031</v>
       </c>
     </row>
-    <row r="613" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="613" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A613" s="1" t="s">
         <v>443</v>
       </c>
@@ -41808,7 +41836,7 @@
         <v>2032</v>
       </c>
     </row>
-    <row r="614" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="614" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A614" s="1" t="s">
         <v>444</v>
       </c>
@@ -41839,7 +41867,7 @@
         <v>2033</v>
       </c>
     </row>
-    <row r="615" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="615" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A615" s="1" t="s">
         <v>2078</v>
       </c>
@@ -41872,7 +41900,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="616" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="616" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A616" s="1" t="s">
         <v>481</v>
       </c>
@@ -41903,7 +41931,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="617" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="617" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A617" s="1" t="s">
         <v>49</v>
       </c>
@@ -41934,7 +41962,7 @@
         <v>2107</v>
       </c>
     </row>
-    <row r="618" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="618" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A618" s="1" t="s">
         <v>2108</v>
       </c>
@@ -42863,9 +42891,11 @@
       </c>
       <c r="H647" s="1"/>
       <c r="I647" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J647" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="J647" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K647" s="1" t="s">
         <v>2076</v>
       </c>
@@ -43372,7 +43402,7 @@
         <v>2105</v>
       </c>
     </row>
-    <row r="664" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="664" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A664" s="1" t="s">
         <v>994</v>
       </c>
@@ -43405,7 +43435,7 @@
         <v>2109</v>
       </c>
     </row>
-    <row r="665" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="665" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A665" s="1" t="s">
         <v>519</v>
       </c>
@@ -43471,7 +43501,7 @@
         <v>1767</v>
       </c>
     </row>
-    <row r="667" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="667" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A667" s="1" t="s">
         <v>2174</v>
       </c>
@@ -44123,9 +44153,11 @@
       </c>
       <c r="H687" s="1"/>
       <c r="I687" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J687" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="J687" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K687" s="1" t="s">
         <v>1075</v>
       </c>
@@ -45164,9 +45196,11 @@
       </c>
       <c r="H720" s="1"/>
       <c r="I720" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J720" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="J720" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K720" s="1" t="s">
         <v>2166</v>
       </c>
@@ -45264,7 +45298,7 @@
         <v>2172</v>
       </c>
     </row>
-    <row r="724" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="724" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A724" s="1" t="s">
         <v>565</v>
       </c>
@@ -46853,7 +46887,7 @@
         <v>2231</v>
       </c>
     </row>
-    <row r="775" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="775" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A775" s="1" t="s">
         <v>566</v>
       </c>
@@ -46884,7 +46918,7 @@
         <v>2234</v>
       </c>
     </row>
-    <row r="776" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="776" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A776" s="1" t="s">
         <v>567</v>
       </c>
@@ -46915,7 +46949,7 @@
         <v>2235</v>
       </c>
     </row>
-    <row r="777" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="777" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A777" s="1" t="s">
         <v>570</v>
       </c>
@@ -47008,7 +47042,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="780" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="780" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A780" s="1" t="s">
         <v>589</v>
       </c>
@@ -47861,7 +47895,7 @@
         <v>2276</v>
       </c>
     </row>
-    <row r="807" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="807" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A807" s="1" t="s">
         <v>1027</v>
       </c>
@@ -49556,9 +49590,11 @@
       </c>
       <c r="H860" s="1"/>
       <c r="I860" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J860" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="J860" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K860" s="1" t="s">
         <v>2352</v>
       </c>
@@ -49587,9 +49623,11 @@
       </c>
       <c r="H861" s="1"/>
       <c r="I861" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="J861" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="J861" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K861" s="1" t="s">
         <v>2353</v>
       </c>
@@ -49649,9 +49687,11 @@
       </c>
       <c r="H863" s="1"/>
       <c r="I863" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J863" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="J863" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K863" s="1" t="s">
         <v>2355</v>
       </c>
@@ -50507,7 +50547,7 @@
         <v>2383</v>
       </c>
     </row>
-    <row r="891" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
+    <row r="891" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A891" s="1" t="s">
         <v>649</v>
       </c>
@@ -50531,7 +50571,7 @@
       </c>
       <c r="H891" s="1"/>
       <c r="I891" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J891" s="1" t="s">
         <v>2975</v>
@@ -50730,7 +50770,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="898" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="898" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A898" s="1" t="s">
         <v>708</v>
       </c>
@@ -51194,9 +51234,11 @@
       </c>
       <c r="H912" s="1"/>
       <c r="I912" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J912" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="J912" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K912" s="1" t="s">
         <v>2419</v>
       </c>
@@ -51921,9 +51963,11 @@
       </c>
       <c r="H935" s="1"/>
       <c r="I935" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J935" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="J935" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K935" s="1" t="s">
         <v>2457</v>
       </c>
@@ -53242,7 +53286,7 @@
         <v>2513</v>
       </c>
     </row>
-    <row r="978" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="978" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A978" s="1" t="s">
         <v>845</v>
       </c>
@@ -53299,9 +53343,11 @@
         <v>2976</v>
       </c>
       <c r="I979" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="J979" s="1"/>
+        <v>4</v>
+      </c>
+      <c r="J979" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K979" s="1" t="s">
         <v>2620</v>
       </c>
@@ -58277,9 +58323,11 @@
       </c>
       <c r="H1137" s="1"/>
       <c r="I1137" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="J1137" s="1"/>
+        <v>4</v>
+      </c>
+      <c r="J1137" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K1137" s="1" t="s">
         <v>2709</v>
       </c>
@@ -59234,7 +59282,7 @@
         <v>2763</v>
       </c>
     </row>
-    <row r="1168" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1168" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1168" s="1" t="s">
         <v>2784</v>
       </c>
@@ -59893,7 +59941,7 @@
         <v>2795</v>
       </c>
     </row>
-    <row r="1189" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1189" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1189" s="1" t="s">
         <v>860</v>
       </c>
@@ -60264,9 +60312,11 @@
       </c>
       <c r="H1200" s="1"/>
       <c r="I1200" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1200" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="J1200" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K1200" s="1" t="s">
         <v>2816</v>
       </c>
@@ -60450,9 +60500,11 @@
       </c>
       <c r="H1206" s="1"/>
       <c r="I1206" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="J1206" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="J1206" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K1206" s="1" t="s">
         <v>2823</v>
       </c>
@@ -61110,7 +61162,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="1228" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1228" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1228" s="1" t="s">
         <v>1015</v>
       </c>
@@ -61417,9 +61469,11 @@
       </c>
       <c r="H1237" s="1"/>
       <c r="I1237" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1237" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="J1237" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K1237" s="1" t="s">
         <v>2865</v>
       </c>
@@ -61773,7 +61827,7 @@
         <v>2750</v>
       </c>
     </row>
-    <row r="1249" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1249" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1249" s="1" t="s">
         <v>899</v>
       </c>
@@ -61804,7 +61858,7 @@
         <v>2886</v>
       </c>
     </row>
-    <row r="1250" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1250" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1250" s="1" t="s">
         <v>900</v>
       </c>
@@ -61835,7 +61889,7 @@
         <v>2887</v>
       </c>
     </row>
-    <row r="1251" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1251" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1251" s="1" t="s">
         <v>938</v>
       </c>
@@ -61866,7 +61920,7 @@
         <v>2888</v>
       </c>
     </row>
-    <row r="1252" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1252" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1252" s="1" t="s">
         <v>901</v>
       </c>
@@ -61899,7 +61953,7 @@
         <v>2889</v>
       </c>
     </row>
-    <row r="1253" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1253" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1253" s="1" t="s">
         <v>902</v>
       </c>
@@ -62087,7 +62141,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="1259" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1259" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1259" s="1" t="s">
         <v>70</v>
       </c>
@@ -62580,9 +62634,11 @@
       </c>
       <c r="H1274" s="1"/>
       <c r="I1274" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J1274" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="J1274" s="1" t="s">
+        <v>2975</v>
+      </c>
       <c r="K1274" s="1" t="s">
         <v>2924</v>
       </c>
@@ -62746,7 +62802,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="1280" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1280" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1280" s="1" t="s">
         <v>1016</v>
       </c>
@@ -62777,7 +62833,7 @@
         <v>2932</v>
       </c>
     </row>
-    <row r="1281" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1281" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1281" s="1" t="s">
         <v>72</v>
       </c>
@@ -63440,7 +63496,7 @@
         <v>2963</v>
       </c>
     </row>
-    <row r="1302" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1302" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A1302" s="1" t="s">
         <v>930</v>
       </c>

</xml_diff>

<commit_message>
new file:   data/chapter2/FRED/subsets/final.csv 	modified:   data/chapter2/FRED/subsets/species.xlsx 	modified:   notebooks/chapter_02/paper-draft.ipynb
</commit_message>
<xml_diff>
--- a/data/chapter2/FRED/subsets/species.xlsx
+++ b/data/chapter2/FRED/subsets/species.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90963425_westernsydney_edu_au/Documents/PhD/code/data/chapter2/FRED/subsets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="897" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A3B0F71-CA45-45D3-8B2E-0D866692243A}"/>
+  <xr:revisionPtr revIDLastSave="900" documentId="8_{81FDA0CF-33C4-43D2-B8CA-CC5F96143B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B8F9DD8-A2C8-4380-9759-3BE4458004B3}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="426" firstSheet="1" activeTab="3" xr2:uid="{A5444074-DC77-415C-A9E2-2BBA8270EAFC}"/>
   </bookViews>
@@ -22418,8 +22418,8 @@
     <col min="1" max="1" width="31" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.1796875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.6328125" customWidth="1"/>
+    <col min="5" max="5" width="15.453125" customWidth="1"/>
     <col min="6" max="6" width="17.26953125" customWidth="1"/>
     <col min="7" max="7" width="17.7265625" customWidth="1"/>
     <col min="8" max="8" width="26.1796875" bestFit="1" customWidth="1"/>

</xml_diff>